<commit_message>
Documentos de «Grupos» paso a paso: ETAPA-2, pendientes (P92, P150, P157, P177, P192 y dos resueltos), inventario de textos con la pantalla nueva y el estado del LEEME
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YEpbunHXM4tST7Mz5ceBJ7
</commit_message>
<xml_diff>
--- a/docs/textos/inventario-textos.xlsx
+++ b/docs/textos/inventario-textos.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Textos" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Textos'!$A$1:$L$803</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Textos'!$A$1:$L$876</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -600,7 +600,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Inventario generado de la versión de prueba 0.66 · 802 textos</t>
+          <t>Inventario generado de la versión de prueba 0.67 · 875 textos</t>
         </is>
       </c>
     </row>
@@ -761,23 +761,23 @@
         </is>
       </c>
       <c r="B21" s="8">
-        <f>COUNTIF(Textos!$B$2:$B$803,A21)</f>
+        <f>COUNTIF(Textos!$B$2:$B$876,A21)</f>
         <v/>
       </c>
       <c r="C21" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$803,A21,Textos!$H$2:$H$803,"Pendiente")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$876,A21,Textos!$H$2:$H$876,"Pendiente")</f>
         <v/>
       </c>
       <c r="D21" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$803,A21,Textos!$H$2:$H$803,"OK")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$876,A21,Textos!$H$2:$H$876,"OK")</f>
         <v/>
       </c>
       <c r="E21" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$803,A21,Textos!$H$2:$H$803,"Cambiar")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$876,A21,Textos!$H$2:$H$876,"Cambiar")</f>
         <v/>
       </c>
       <c r="F21" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$803,A21,Textos!$H$2:$H$803,"Quitar")+COUNTIFS(Textos!$B$2:$B$803,A21,Textos!$H$2:$H$803,"Duda")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$876,A21,Textos!$H$2:$H$876,"Quitar")+COUNTIFS(Textos!$B$2:$B$876,A21,Textos!$H$2:$H$876,"Duda")</f>
         <v/>
       </c>
     </row>
@@ -788,23 +788,23 @@
         </is>
       </c>
       <c r="B22" s="8">
-        <f>COUNTIF(Textos!$B$2:$B$803,A22)</f>
+        <f>COUNTIF(Textos!$B$2:$B$876,A22)</f>
         <v/>
       </c>
       <c r="C22" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$803,A22,Textos!$H$2:$H$803,"Pendiente")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$876,A22,Textos!$H$2:$H$876,"Pendiente")</f>
         <v/>
       </c>
       <c r="D22" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$803,A22,Textos!$H$2:$H$803,"OK")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$876,A22,Textos!$H$2:$H$876,"OK")</f>
         <v/>
       </c>
       <c r="E22" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$803,A22,Textos!$H$2:$H$803,"Cambiar")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$876,A22,Textos!$H$2:$H$876,"Cambiar")</f>
         <v/>
       </c>
       <c r="F22" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$803,A22,Textos!$H$2:$H$803,"Quitar")+COUNTIFS(Textos!$B$2:$B$803,A22,Textos!$H$2:$H$803,"Duda")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$876,A22,Textos!$H$2:$H$876,"Quitar")+COUNTIFS(Textos!$B$2:$B$876,A22,Textos!$H$2:$H$876,"Duda")</f>
         <v/>
       </c>
     </row>
@@ -815,23 +815,23 @@
         </is>
       </c>
       <c r="B23" s="8">
-        <f>COUNTIF(Textos!$B$2:$B$803,A23)</f>
+        <f>COUNTIF(Textos!$B$2:$B$876,A23)</f>
         <v/>
       </c>
       <c r="C23" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$803,A23,Textos!$H$2:$H$803,"Pendiente")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$876,A23,Textos!$H$2:$H$876,"Pendiente")</f>
         <v/>
       </c>
       <c r="D23" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$803,A23,Textos!$H$2:$H$803,"OK")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$876,A23,Textos!$H$2:$H$876,"OK")</f>
         <v/>
       </c>
       <c r="E23" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$803,A23,Textos!$H$2:$H$803,"Cambiar")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$876,A23,Textos!$H$2:$H$876,"Cambiar")</f>
         <v/>
       </c>
       <c r="F23" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$803,A23,Textos!$H$2:$H$803,"Quitar")+COUNTIFS(Textos!$B$2:$B$803,A23,Textos!$H$2:$H$803,"Duda")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$876,A23,Textos!$H$2:$H$876,"Quitar")+COUNTIFS(Textos!$B$2:$B$876,A23,Textos!$H$2:$H$876,"Duda")</f>
         <v/>
       </c>
     </row>
@@ -842,23 +842,23 @@
         </is>
       </c>
       <c r="B24" s="8">
-        <f>COUNTIF(Textos!$B$2:$B$803,A24)</f>
+        <f>COUNTIF(Textos!$B$2:$B$876,A24)</f>
         <v/>
       </c>
       <c r="C24" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$803,A24,Textos!$H$2:$H$803,"Pendiente")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$876,A24,Textos!$H$2:$H$876,"Pendiente")</f>
         <v/>
       </c>
       <c r="D24" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$803,A24,Textos!$H$2:$H$803,"OK")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$876,A24,Textos!$H$2:$H$876,"OK")</f>
         <v/>
       </c>
       <c r="E24" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$803,A24,Textos!$H$2:$H$803,"Cambiar")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$876,A24,Textos!$H$2:$H$876,"Cambiar")</f>
         <v/>
       </c>
       <c r="F24" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$803,A24,Textos!$H$2:$H$803,"Quitar")+COUNTIFS(Textos!$B$2:$B$803,A24,Textos!$H$2:$H$803,"Duda")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$876,A24,Textos!$H$2:$H$876,"Quitar")+COUNTIFS(Textos!$B$2:$B$876,A24,Textos!$H$2:$H$876,"Duda")</f>
         <v/>
       </c>
     </row>
@@ -869,23 +869,23 @@
         </is>
       </c>
       <c r="B25" s="8">
-        <f>COUNTIF(Textos!$B$2:$B$803,A25)</f>
+        <f>COUNTIF(Textos!$B$2:$B$876,A25)</f>
         <v/>
       </c>
       <c r="C25" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$803,A25,Textos!$H$2:$H$803,"Pendiente")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$876,A25,Textos!$H$2:$H$876,"Pendiente")</f>
         <v/>
       </c>
       <c r="D25" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$803,A25,Textos!$H$2:$H$803,"OK")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$876,A25,Textos!$H$2:$H$876,"OK")</f>
         <v/>
       </c>
       <c r="E25" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$803,A25,Textos!$H$2:$H$803,"Cambiar")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$876,A25,Textos!$H$2:$H$876,"Cambiar")</f>
         <v/>
       </c>
       <c r="F25" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$803,A25,Textos!$H$2:$H$803,"Quitar")+COUNTIFS(Textos!$B$2:$B$803,A25,Textos!$H$2:$H$803,"Duda")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$876,A25,Textos!$H$2:$H$876,"Quitar")+COUNTIFS(Textos!$B$2:$B$876,A25,Textos!$H$2:$H$876,"Duda")</f>
         <v/>
       </c>
     </row>
@@ -896,23 +896,23 @@
         </is>
       </c>
       <c r="B26" s="8">
-        <f>COUNTIF(Textos!$B$2:$B$803,A26)</f>
+        <f>COUNTIF(Textos!$B$2:$B$876,A26)</f>
         <v/>
       </c>
       <c r="C26" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$803,A26,Textos!$H$2:$H$803,"Pendiente")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$876,A26,Textos!$H$2:$H$876,"Pendiente")</f>
         <v/>
       </c>
       <c r="D26" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$803,A26,Textos!$H$2:$H$803,"OK")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$876,A26,Textos!$H$2:$H$876,"OK")</f>
         <v/>
       </c>
       <c r="E26" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$803,A26,Textos!$H$2:$H$803,"Cambiar")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$876,A26,Textos!$H$2:$H$876,"Cambiar")</f>
         <v/>
       </c>
       <c r="F26" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$803,A26,Textos!$H$2:$H$803,"Quitar")+COUNTIFS(Textos!$B$2:$B$803,A26,Textos!$H$2:$H$803,"Duda")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$876,A26,Textos!$H$2:$H$876,"Quitar")+COUNTIFS(Textos!$B$2:$B$876,A26,Textos!$H$2:$H$876,"Duda")</f>
         <v/>
       </c>
     </row>
@@ -923,23 +923,23 @@
         </is>
       </c>
       <c r="B27" s="8">
-        <f>COUNTIF(Textos!$B$2:$B$803,A27)</f>
+        <f>COUNTIF(Textos!$B$2:$B$876,A27)</f>
         <v/>
       </c>
       <c r="C27" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$803,A27,Textos!$H$2:$H$803,"Pendiente")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$876,A27,Textos!$H$2:$H$876,"Pendiente")</f>
         <v/>
       </c>
       <c r="D27" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$803,A27,Textos!$H$2:$H$803,"OK")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$876,A27,Textos!$H$2:$H$876,"OK")</f>
         <v/>
       </c>
       <c r="E27" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$803,A27,Textos!$H$2:$H$803,"Cambiar")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$876,A27,Textos!$H$2:$H$876,"Cambiar")</f>
         <v/>
       </c>
       <c r="F27" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$803,A27,Textos!$H$2:$H$803,"Quitar")+COUNTIFS(Textos!$B$2:$B$803,A27,Textos!$H$2:$H$803,"Duda")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$876,A27,Textos!$H$2:$H$876,"Quitar")+COUNTIFS(Textos!$B$2:$B$876,A27,Textos!$H$2:$H$876,"Duda")</f>
         <v/>
       </c>
     </row>
@@ -950,23 +950,23 @@
         </is>
       </c>
       <c r="B28" s="8">
-        <f>COUNTIF(Textos!$B$2:$B$803,A28)</f>
+        <f>COUNTIF(Textos!$B$2:$B$876,A28)</f>
         <v/>
       </c>
       <c r="C28" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$803,A28,Textos!$H$2:$H$803,"Pendiente")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$876,A28,Textos!$H$2:$H$876,"Pendiente")</f>
         <v/>
       </c>
       <c r="D28" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$803,A28,Textos!$H$2:$H$803,"OK")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$876,A28,Textos!$H$2:$H$876,"OK")</f>
         <v/>
       </c>
       <c r="E28" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$803,A28,Textos!$H$2:$H$803,"Cambiar")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$876,A28,Textos!$H$2:$H$876,"Cambiar")</f>
         <v/>
       </c>
       <c r="F28" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$803,A28,Textos!$H$2:$H$803,"Quitar")+COUNTIFS(Textos!$B$2:$B$803,A28,Textos!$H$2:$H$803,"Duda")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$876,A28,Textos!$H$2:$H$876,"Quitar")+COUNTIFS(Textos!$B$2:$B$876,A28,Textos!$H$2:$H$876,"Duda")</f>
         <v/>
       </c>
     </row>
@@ -977,23 +977,23 @@
         </is>
       </c>
       <c r="B29" s="8">
-        <f>COUNTIF(Textos!$B$2:$B$803,A29)</f>
+        <f>COUNTIF(Textos!$B$2:$B$876,A29)</f>
         <v/>
       </c>
       <c r="C29" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$803,A29,Textos!$H$2:$H$803,"Pendiente")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$876,A29,Textos!$H$2:$H$876,"Pendiente")</f>
         <v/>
       </c>
       <c r="D29" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$803,A29,Textos!$H$2:$H$803,"OK")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$876,A29,Textos!$H$2:$H$876,"OK")</f>
         <v/>
       </c>
       <c r="E29" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$803,A29,Textos!$H$2:$H$803,"Cambiar")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$876,A29,Textos!$H$2:$H$876,"Cambiar")</f>
         <v/>
       </c>
       <c r="F29" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$803,A29,Textos!$H$2:$H$803,"Quitar")+COUNTIFS(Textos!$B$2:$B$803,A29,Textos!$H$2:$H$803,"Duda")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$876,A29,Textos!$H$2:$H$876,"Quitar")+COUNTIFS(Textos!$B$2:$B$876,A29,Textos!$H$2:$H$876,"Duda")</f>
         <v/>
       </c>
     </row>
@@ -1004,23 +1004,23 @@
         </is>
       </c>
       <c r="B30" s="8">
-        <f>COUNTIF(Textos!$B$2:$B$803,A30)</f>
+        <f>COUNTIF(Textos!$B$2:$B$876,A30)</f>
         <v/>
       </c>
       <c r="C30" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$803,A30,Textos!$H$2:$H$803,"Pendiente")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$876,A30,Textos!$H$2:$H$876,"Pendiente")</f>
         <v/>
       </c>
       <c r="D30" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$803,A30,Textos!$H$2:$H$803,"OK")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$876,A30,Textos!$H$2:$H$876,"OK")</f>
         <v/>
       </c>
       <c r="E30" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$803,A30,Textos!$H$2:$H$803,"Cambiar")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$876,A30,Textos!$H$2:$H$876,"Cambiar")</f>
         <v/>
       </c>
       <c r="F30" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$803,A30,Textos!$H$2:$H$803,"Quitar")+COUNTIFS(Textos!$B$2:$B$803,A30,Textos!$H$2:$H$803,"Duda")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$876,A30,Textos!$H$2:$H$876,"Quitar")+COUNTIFS(Textos!$B$2:$B$876,A30,Textos!$H$2:$H$876,"Duda")</f>
         <v/>
       </c>
     </row>
@@ -1031,23 +1031,23 @@
         </is>
       </c>
       <c r="B31" s="8">
-        <f>COUNTIF(Textos!$B$2:$B$803,A31)</f>
+        <f>COUNTIF(Textos!$B$2:$B$876,A31)</f>
         <v/>
       </c>
       <c r="C31" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$803,A31,Textos!$H$2:$H$803,"Pendiente")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$876,A31,Textos!$H$2:$H$876,"Pendiente")</f>
         <v/>
       </c>
       <c r="D31" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$803,A31,Textos!$H$2:$H$803,"OK")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$876,A31,Textos!$H$2:$H$876,"OK")</f>
         <v/>
       </c>
       <c r="E31" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$803,A31,Textos!$H$2:$H$803,"Cambiar")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$876,A31,Textos!$H$2:$H$876,"Cambiar")</f>
         <v/>
       </c>
       <c r="F31" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$803,A31,Textos!$H$2:$H$803,"Quitar")+COUNTIFS(Textos!$B$2:$B$803,A31,Textos!$H$2:$H$803,"Duda")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$876,A31,Textos!$H$2:$H$876,"Quitar")+COUNTIFS(Textos!$B$2:$B$876,A31,Textos!$H$2:$H$876,"Duda")</f>
         <v/>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L803"/>
+  <dimension ref="A1:L876"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -41180,12 +41180,12 @@
       </c>
       <c r="B801" s="15" t="inlineStr">
         <is>
-          <t>Reposición de tu credencial</t>
+          <t>Grupos (personal)</t>
         </is>
       </c>
       <c r="C801" s="15" t="inlineStr">
         <is>
-          <t>Resultado</t>
+          <t>Grupos</t>
         </is>
       </c>
       <c r="D801" s="15" t="inlineStr">
@@ -41195,12 +41195,12 @@
       </c>
       <c r="E801" s="15" t="inlineStr">
         <is>
-          <t>Al pedirla o al cargar el acta corregida</t>
+          <t>Siempre</t>
         </is>
       </c>
       <c r="F801" s="15" t="inlineStr">
         <is>
-          <t>Recibimos tu solicitud de reposición · Recibimos tu acta corregida</t>
+          <t>Grupos</t>
         </is>
       </c>
       <c r="G801" s="13" t="inlineStr"/>
@@ -41213,12 +41213,12 @@
       <c r="J801" s="15" t="inlineStr"/>
       <c r="K801" s="16" t="inlineStr">
         <is>
-          <t>Persona solicitante</t>
+          <t>Personal de la Secretaría</t>
         </is>
       </c>
       <c r="L801" s="16" t="inlineStr">
         <is>
-          <t>Código del sitio (sitio/app/reposicion.js)</t>
+          <t>Página (sitio/grupos.html)</t>
         </is>
       </c>
     </row>
@@ -41230,27 +41230,27 @@
       </c>
       <c r="B802" s="12" t="inlineStr">
         <is>
-          <t>Reposición de tu credencial</t>
+          <t>Grupos (personal)</t>
         </is>
       </c>
       <c r="C802" s="12" t="inlineStr">
         <is>
-          <t>Resultado</t>
+          <t>Grupos</t>
         </is>
       </c>
       <c r="D802" s="12" t="inlineStr">
         <is>
-          <t>Pasos</t>
+          <t>Introducción</t>
         </is>
       </c>
       <c r="E802" s="12" t="inlineStr">
         <is>
-          <t>Al pedirla</t>
+          <t>Siempre</t>
         </is>
       </c>
       <c r="F802" s="12" t="inlineStr">
         <is>
-          <t>La Secretaría revisa tu acta. · Te indica en «Mis trámites» si debes corregir algo o, si está completa, cuánto pagar. · Pagas la cuota de reposición y recoges tu credencial en la oficina del Vivero Nezahualcóyotl, con el mismo número y la misma vigencia.</t>
+          <t>Cargando los grupos…</t>
         </is>
       </c>
       <c r="G802" s="13" t="inlineStr"/>
@@ -41260,15 +41260,19 @@
         </is>
       </c>
       <c r="I802" s="13" t="inlineStr"/>
-      <c r="J802" s="12" t="inlineStr"/>
+      <c r="J802" s="17" t="inlineStr">
+        <is>
+          <t>Texto momentáneo mientras cargan los datos.</t>
+        </is>
+      </c>
       <c r="K802" s="14" t="inlineStr">
         <is>
-          <t>Persona solicitante</t>
+          <t>Personal de la Secretaría</t>
         </is>
       </c>
       <c r="L802" s="14" t="inlineStr">
         <is>
-          <t>Código del sitio (sitio/app/reposicion.js)</t>
+          <t>Página (sitio/grupos.html)</t>
         </is>
       </c>
     </row>
@@ -41280,27 +41284,27 @@
       </c>
       <c r="B803" s="15" t="inlineStr">
         <is>
-          <t>Reposición de tu credencial</t>
+          <t>Grupos (personal)</t>
         </is>
       </c>
       <c r="C803" s="15" t="inlineStr">
         <is>
-          <t>Acreditación</t>
+          <t>Grupos</t>
         </is>
       </c>
       <c r="D803" s="15" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Botón o enlace</t>
         </is>
       </c>
       <c r="E803" s="15" t="inlineStr">
         <is>
-          <t>Credencial del sistema que todavía no se entrega</t>
+          <t>Siempre</t>
         </is>
       </c>
       <c r="F803" s="15" t="inlineStr">
         <is>
-          <t>Tu credencial todavía no se te entrega: recógela en la oficina del Vivero. La reposición es para una credencial que ya recibiste y perdiste o te robaron.</t>
+          <t>Ver los grupos programados</t>
         </is>
       </c>
       <c r="G803" s="13" t="inlineStr"/>
@@ -41313,18 +41317,3668 @@
       <c r="J803" s="15" t="inlineStr"/>
       <c r="K803" s="16" t="inlineStr">
         <is>
-          <t>Persona solicitante</t>
+          <t>Personal de la Secretaría</t>
         </is>
       </c>
       <c r="L803" s="16" t="inlineStr">
         <is>
+          <t>Página (sitio/grupos.html)</t>
+        </is>
+      </c>
+    </row>
+    <row r="804">
+      <c r="A804" s="12" t="inlineStr">
+        <is>
+          <t>T803</t>
+        </is>
+      </c>
+      <c r="B804" s="12" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C804" s="12" t="inlineStr">
+        <is>
+          <t>Armar un grupo</t>
+        </is>
+      </c>
+      <c r="D804" s="12" t="inlineStr">
+        <is>
+          <t>Subtítulo</t>
+        </is>
+      </c>
+      <c r="E804" s="12" t="inlineStr">
+        <is>
+          <t>Siempre</t>
+        </is>
+      </c>
+      <c r="F804" s="12" t="inlineStr">
+        <is>
+          <t>Armar un grupo</t>
+        </is>
+      </c>
+      <c r="G804" s="13" t="inlineStr"/>
+      <c r="H804" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I804" s="13" t="inlineStr"/>
+      <c r="J804" s="12" t="inlineStr"/>
+      <c r="K804" s="14" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L804" s="14" t="inlineStr">
+        <is>
+          <t>Página (sitio/grupos.html)</t>
+        </is>
+      </c>
+    </row>
+    <row r="805">
+      <c r="A805" s="15" t="inlineStr">
+        <is>
+          <t>T804</t>
+        </is>
+      </c>
+      <c r="B805" s="15" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C805" s="15" t="inlineStr">
+        <is>
+          <t>El curso</t>
+        </is>
+      </c>
+      <c r="D805" s="15" t="inlineStr">
+        <is>
+          <t>Subtítulo</t>
+        </is>
+      </c>
+      <c r="E805" s="15" t="inlineStr">
+        <is>
+          <t>Siempre</t>
+        </is>
+      </c>
+      <c r="F805" s="15" t="inlineStr">
+        <is>
+          <t>¿Para qué curso?</t>
+        </is>
+      </c>
+      <c r="G805" s="13" t="inlineStr"/>
+      <c r="H805" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I805" s="13" t="inlineStr"/>
+      <c r="J805" s="15" t="inlineStr"/>
+      <c r="K805" s="16" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L805" s="16" t="inlineStr">
+        <is>
+          <t>Página (sitio/grupos.html)</t>
+        </is>
+      </c>
+    </row>
+    <row r="806">
+      <c r="A806" s="12" t="inlineStr">
+        <is>
+          <t>T805</t>
+        </is>
+      </c>
+      <c r="B806" s="12" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C806" s="12" t="inlineStr">
+        <is>
+          <t>El curso</t>
+        </is>
+      </c>
+      <c r="D806" s="12" t="inlineStr">
+        <is>
+          <t>Introducción</t>
+        </is>
+      </c>
+      <c r="E806" s="12" t="inlineStr">
+        <is>
+          <t>Siempre</t>
+        </is>
+      </c>
+      <c r="F806" s="12" t="inlineStr">
+        <is>
+          <t>Cada curso arma sus grupos por separado: nunca se mezclan.</t>
+        </is>
+      </c>
+      <c r="G806" s="13" t="inlineStr"/>
+      <c r="H806" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I806" s="13" t="inlineStr"/>
+      <c r="J806" s="12" t="inlineStr"/>
+      <c r="K806" s="14" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L806" s="14" t="inlineStr">
+        <is>
+          <t>Página (sitio/grupos.html)</t>
+        </is>
+      </c>
+    </row>
+    <row r="807">
+      <c r="A807" s="15" t="inlineStr">
+        <is>
+          <t>T806</t>
+        </is>
+      </c>
+      <c r="B807" s="15" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C807" s="15" t="inlineStr">
+        <is>
+          <t>El curso</t>
+        </is>
+      </c>
+      <c r="D807" s="15" t="inlineStr">
+        <is>
+          <t>Opción</t>
+        </is>
+      </c>
+      <c r="E807" s="15" t="inlineStr">
+        <is>
+          <t>Siempre</t>
+        </is>
+      </c>
+      <c r="F807" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Poda y derribo · nueva — </t>
+        </is>
+      </c>
+      <c r="G807" s="13" t="inlineStr"/>
+      <c r="H807" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I807" s="13" t="inlineStr"/>
+      <c r="J807" s="15" t="inlineStr"/>
+      <c r="K807" s="16" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L807" s="16" t="inlineStr">
+        <is>
+          <t>Página (sitio/grupos.html)</t>
+        </is>
+      </c>
+    </row>
+    <row r="808">
+      <c r="A808" s="12" t="inlineStr">
+        <is>
+          <t>T807</t>
+        </is>
+      </c>
+      <c r="B808" s="12" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C808" s="12" t="inlineStr">
+        <is>
+          <t>El curso</t>
+        </is>
+      </c>
+      <c r="D808" s="12" t="inlineStr">
+        <is>
+          <t>Opción</t>
+        </is>
+      </c>
+      <c r="E808" s="12" t="inlineStr">
+        <is>
+          <t>Siempre</t>
+        </is>
+      </c>
+      <c r="F808" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Poda y derribo · renovación — </t>
+        </is>
+      </c>
+      <c r="G808" s="13" t="inlineStr"/>
+      <c r="H808" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I808" s="13" t="inlineStr"/>
+      <c r="J808" s="12" t="inlineStr"/>
+      <c r="K808" s="14" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L808" s="14" t="inlineStr">
+        <is>
+          <t>Página (sitio/grupos.html)</t>
+        </is>
+      </c>
+    </row>
+    <row r="809">
+      <c r="A809" s="15" t="inlineStr">
+        <is>
+          <t>T808</t>
+        </is>
+      </c>
+      <c r="B809" s="15" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C809" s="15" t="inlineStr">
+        <is>
+          <t>El curso</t>
+        </is>
+      </c>
+      <c r="D809" s="15" t="inlineStr">
+        <is>
+          <t>Opción</t>
+        </is>
+      </c>
+      <c r="E809" s="15" t="inlineStr">
+        <is>
+          <t>Siempre</t>
+        </is>
+      </c>
+      <c r="F809" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dictaminador técnico · nueva — </t>
+        </is>
+      </c>
+      <c r="G809" s="13" t="inlineStr"/>
+      <c r="H809" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I809" s="13" t="inlineStr"/>
+      <c r="J809" s="15" t="inlineStr"/>
+      <c r="K809" s="16" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L809" s="16" t="inlineStr">
+        <is>
+          <t>Página (sitio/grupos.html)</t>
+        </is>
+      </c>
+    </row>
+    <row r="810">
+      <c r="A810" s="12" t="inlineStr">
+        <is>
+          <t>T809</t>
+        </is>
+      </c>
+      <c r="B810" s="12" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C810" s="12" t="inlineStr">
+        <is>
+          <t>El curso</t>
+        </is>
+      </c>
+      <c r="D810" s="12" t="inlineStr">
+        <is>
+          <t>Opción</t>
+        </is>
+      </c>
+      <c r="E810" s="12" t="inlineStr">
+        <is>
+          <t>Siempre</t>
+        </is>
+      </c>
+      <c r="F810" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dictaminador técnico · renovación — </t>
+        </is>
+      </c>
+      <c r="G810" s="13" t="inlineStr"/>
+      <c r="H810" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I810" s="13" t="inlineStr"/>
+      <c r="J810" s="12" t="inlineStr"/>
+      <c r="K810" s="14" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L810" s="14" t="inlineStr">
+        <is>
+          <t>Página (sitio/grupos.html)</t>
+        </is>
+      </c>
+    </row>
+    <row r="811">
+      <c r="A811" s="15" t="inlineStr">
+        <is>
+          <t>T810</t>
+        </is>
+      </c>
+      <c r="B811" s="15" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C811" s="15" t="inlineStr">
+        <is>
+          <t>El curso</t>
+        </is>
+      </c>
+      <c r="D811" s="15" t="inlineStr">
+        <is>
+          <t>Botón o enlace</t>
+        </is>
+      </c>
+      <c r="E811" s="15" t="inlineStr">
+        <is>
+          <t>Siempre</t>
+        </is>
+      </c>
+      <c r="F811" s="15" t="inlineStr">
+        <is>
+          <t>Siguiente</t>
+        </is>
+      </c>
+      <c r="G811" s="13" t="inlineStr"/>
+      <c r="H811" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I811" s="13" t="inlineStr"/>
+      <c r="J811" s="15" t="inlineStr"/>
+      <c r="K811" s="16" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L811" s="16" t="inlineStr">
+        <is>
+          <t>Página (sitio/grupos.html)</t>
+        </is>
+      </c>
+    </row>
+    <row r="812">
+      <c r="A812" s="12" t="inlineStr">
+        <is>
+          <t>T811</t>
+        </is>
+      </c>
+      <c r="B812" s="12" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C812" s="12" t="inlineStr">
+        <is>
+          <t>La semana</t>
+        </is>
+      </c>
+      <c r="D812" s="12" t="inlineStr">
+        <is>
+          <t>Subtítulo</t>
+        </is>
+      </c>
+      <c r="E812" s="12" t="inlineStr">
+        <is>
+          <t>Siempre</t>
+        </is>
+      </c>
+      <c r="F812" s="12" t="inlineStr">
+        <is>
+          <t>¿Qué semana?</t>
+        </is>
+      </c>
+      <c r="G812" s="13" t="inlineStr"/>
+      <c r="H812" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I812" s="13" t="inlineStr"/>
+      <c r="J812" s="12" t="inlineStr"/>
+      <c r="K812" s="14" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L812" s="14" t="inlineStr">
+        <is>
+          <t>Página (sitio/grupos.html)</t>
+        </is>
+      </c>
+    </row>
+    <row r="813">
+      <c r="A813" s="15" t="inlineStr">
+        <is>
+          <t>T812</t>
+        </is>
+      </c>
+      <c r="B813" s="15" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C813" s="15" t="inlineStr">
+        <is>
+          <t>La semana</t>
+        </is>
+      </c>
+      <c r="D813" s="15" t="inlineStr">
+        <is>
+          <t>Texto</t>
+        </is>
+      </c>
+      <c r="E813" s="15" t="inlineStr">
+        <is>
+          <t>Siempre</t>
+        </is>
+      </c>
+      <c r="F813" s="15" t="inlineStr">
+        <is>
+          <t>Semana elegida</t>
+        </is>
+      </c>
+      <c r="G813" s="13" t="inlineStr"/>
+      <c r="H813" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I813" s="13" t="inlineStr"/>
+      <c r="J813" s="15" t="inlineStr"/>
+      <c r="K813" s="16" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L813" s="16" t="inlineStr">
+        <is>
+          <t>Página (sitio/grupos.html)</t>
+        </is>
+      </c>
+    </row>
+    <row r="814">
+      <c r="A814" s="12" t="inlineStr">
+        <is>
+          <t>T813</t>
+        </is>
+      </c>
+      <c r="B814" s="12" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C814" s="12" t="inlineStr">
+        <is>
+          <t>La semana</t>
+        </is>
+      </c>
+      <c r="D814" s="12" t="inlineStr">
+        <is>
+          <t>Texto</t>
+        </is>
+      </c>
+      <c r="E814" s="12" t="inlineStr">
+        <is>
+          <t>Siempre</t>
+        </is>
+      </c>
+      <c r="F814" s="12" t="inlineStr">
+        <is>
+          <t>Ninguna todavía</t>
+        </is>
+      </c>
+      <c r="G814" s="13" t="inlineStr"/>
+      <c r="H814" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I814" s="13" t="inlineStr"/>
+      <c r="J814" s="12" t="inlineStr"/>
+      <c r="K814" s="14" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L814" s="14" t="inlineStr">
+        <is>
+          <t>Página (sitio/grupos.html)</t>
+        </is>
+      </c>
+    </row>
+    <row r="815">
+      <c r="A815" s="15" t="inlineStr">
+        <is>
+          <t>T814</t>
+        </is>
+      </c>
+      <c r="B815" s="15" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C815" s="15" t="inlineStr">
+        <is>
+          <t>La semana</t>
+        </is>
+      </c>
+      <c r="D815" s="15" t="inlineStr">
+        <is>
+          <t>Pregunta</t>
+        </is>
+      </c>
+      <c r="E815" s="15" t="inlineStr">
+        <is>
+          <t>Siempre</t>
+        </is>
+      </c>
+      <c r="F815" s="15" t="inlineStr">
+        <is>
+          <t>Primer día del curso</t>
+        </is>
+      </c>
+      <c r="G815" s="13" t="inlineStr"/>
+      <c r="H815" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I815" s="13" t="inlineStr"/>
+      <c r="J815" s="15" t="inlineStr"/>
+      <c r="K815" s="16" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L815" s="16" t="inlineStr">
+        <is>
+          <t>Página (sitio/grupos.html)</t>
+        </is>
+      </c>
+    </row>
+    <row r="816">
+      <c r="A816" s="12" t="inlineStr">
+        <is>
+          <t>T815</t>
+        </is>
+      </c>
+      <c r="B816" s="12" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C816" s="12" t="inlineStr">
+        <is>
+          <t>La semana</t>
+        </is>
+      </c>
+      <c r="D816" s="12" t="inlineStr">
+        <is>
+          <t>Ayuda</t>
+        </is>
+      </c>
+      <c r="E816" s="12" t="inlineStr">
+        <is>
+          <t>Siempre</t>
+        </is>
+      </c>
+      <c r="F816" s="12" t="inlineStr">
+        <is>
+          <t>Se llena al elegir la semana en el calendario.</t>
+        </is>
+      </c>
+      <c r="G816" s="13" t="inlineStr"/>
+      <c r="H816" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I816" s="13" t="inlineStr"/>
+      <c r="J816" s="12" t="inlineStr"/>
+      <c r="K816" s="14" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L816" s="14" t="inlineStr">
+        <is>
+          <t>Página (sitio/grupos.html)</t>
+        </is>
+      </c>
+    </row>
+    <row r="817">
+      <c r="A817" s="15" t="inlineStr">
+        <is>
+          <t>T816</t>
+        </is>
+      </c>
+      <c r="B817" s="15" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C817" s="15" t="inlineStr">
+        <is>
+          <t>La semana</t>
+        </is>
+      </c>
+      <c r="D817" s="15" t="inlineStr">
+        <is>
+          <t>Texto</t>
+        </is>
+      </c>
+      <c r="E817" s="15" t="inlineStr">
+        <is>
+          <t>Siempre</t>
+        </is>
+      </c>
+      <c r="F817" s="15" t="inlineStr">
+        <is>
+          <t>Semana libre: toque «Libre» para elegirla</t>
+        </is>
+      </c>
+      <c r="G817" s="13" t="inlineStr"/>
+      <c r="H817" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I817" s="13" t="inlineStr"/>
+      <c r="J817" s="15" t="inlineStr"/>
+      <c r="K817" s="16" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L817" s="16" t="inlineStr">
+        <is>
+          <t>Página (sitio/grupos.html)</t>
+        </is>
+      </c>
+    </row>
+    <row r="818">
+      <c r="A818" s="12" t="inlineStr">
+        <is>
+          <t>T817</t>
+        </is>
+      </c>
+      <c r="B818" s="12" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C818" s="12" t="inlineStr">
+        <is>
+          <t>La semana</t>
+        </is>
+      </c>
+      <c r="D818" s="12" t="inlineStr">
+        <is>
+          <t>Texto</t>
+        </is>
+      </c>
+      <c r="E818" s="12" t="inlineStr">
+        <is>
+          <t>Siempre</t>
+        </is>
+      </c>
+      <c r="F818" s="12" t="inlineStr">
+        <is>
+          <t>El grupo nuevo</t>
+        </is>
+      </c>
+      <c r="G818" s="13" t="inlineStr"/>
+      <c r="H818" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I818" s="13" t="inlineStr"/>
+      <c r="J818" s="12" t="inlineStr"/>
+      <c r="K818" s="14" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L818" s="14" t="inlineStr">
+        <is>
+          <t>Página (sitio/grupos.html)</t>
+        </is>
+      </c>
+    </row>
+    <row r="819">
+      <c r="A819" s="15" t="inlineStr">
+        <is>
+          <t>T818</t>
+        </is>
+      </c>
+      <c r="B819" s="15" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C819" s="15" t="inlineStr">
+        <is>
+          <t>La semana</t>
+        </is>
+      </c>
+      <c r="D819" s="15" t="inlineStr">
+        <is>
+          <t>Texto</t>
+        </is>
+      </c>
+      <c r="E819" s="15" t="inlineStr">
+        <is>
+          <t>Siempre</t>
+        </is>
+      </c>
+      <c r="F819" s="15" t="inlineStr">
+        <is>
+          <t>Grupo por confirmar</t>
+        </is>
+      </c>
+      <c r="G819" s="13" t="inlineStr"/>
+      <c r="H819" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I819" s="13" t="inlineStr"/>
+      <c r="J819" s="15" t="inlineStr"/>
+      <c r="K819" s="16" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L819" s="16" t="inlineStr">
+        <is>
+          <t>Página (sitio/grupos.html)</t>
+        </is>
+      </c>
+    </row>
+    <row r="820">
+      <c r="A820" s="12" t="inlineStr">
+        <is>
+          <t>T819</t>
+        </is>
+      </c>
+      <c r="B820" s="12" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C820" s="12" t="inlineStr">
+        <is>
+          <t>La semana</t>
+        </is>
+      </c>
+      <c r="D820" s="12" t="inlineStr">
+        <is>
+          <t>Texto</t>
+        </is>
+      </c>
+      <c r="E820" s="12" t="inlineStr">
+        <is>
+          <t>Siempre</t>
+        </is>
+      </c>
+      <c r="F820" s="12" t="inlineStr">
+        <is>
+          <t>Grupo confirmado</t>
+        </is>
+      </c>
+      <c r="G820" s="13" t="inlineStr"/>
+      <c r="H820" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I820" s="13" t="inlineStr"/>
+      <c r="J820" s="12" t="inlineStr"/>
+      <c r="K820" s="14" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L820" s="14" t="inlineStr">
+        <is>
+          <t>Página (sitio/grupos.html)</t>
+        </is>
+      </c>
+    </row>
+    <row r="821">
+      <c r="A821" s="15" t="inlineStr">
+        <is>
+          <t>T820</t>
+        </is>
+      </c>
+      <c r="B821" s="15" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C821" s="15" t="inlineStr">
+        <is>
+          <t>La semana</t>
+        </is>
+      </c>
+      <c r="D821" s="15" t="inlineStr">
+        <is>
+          <t>Texto</t>
+        </is>
+      </c>
+      <c r="E821" s="15" t="inlineStr">
+        <is>
+          <t>Siempre</t>
+        </is>
+      </c>
+      <c r="F821" s="15" t="inlineStr">
+        <is>
+          <t>Grupo en curso</t>
+        </is>
+      </c>
+      <c r="G821" s="13" t="inlineStr"/>
+      <c r="H821" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I821" s="13" t="inlineStr"/>
+      <c r="J821" s="15" t="inlineStr"/>
+      <c r="K821" s="16" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L821" s="16" t="inlineStr">
+        <is>
+          <t>Página (sitio/grupos.html)</t>
+        </is>
+      </c>
+    </row>
+    <row r="822">
+      <c r="A822" s="12" t="inlineStr">
+        <is>
+          <t>T821</t>
+        </is>
+      </c>
+      <c r="B822" s="12" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C822" s="12" t="inlineStr">
+        <is>
+          <t>La semana</t>
+        </is>
+      </c>
+      <c r="D822" s="12" t="inlineStr">
+        <is>
+          <t>Texto</t>
+        </is>
+      </c>
+      <c r="E822" s="12" t="inlineStr">
+        <is>
+          <t>Siempre</t>
+        </is>
+      </c>
+      <c r="F822" s="12" t="inlineStr">
+        <is>
+          <t>Grupo que ya terminó</t>
+        </is>
+      </c>
+      <c r="G822" s="13" t="inlineStr"/>
+      <c r="H822" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I822" s="13" t="inlineStr"/>
+      <c r="J822" s="12" t="inlineStr"/>
+      <c r="K822" s="14" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L822" s="14" t="inlineStr">
+        <is>
+          <t>Página (sitio/grupos.html)</t>
+        </is>
+      </c>
+    </row>
+    <row r="823">
+      <c r="A823" s="15" t="inlineStr">
+        <is>
+          <t>T822</t>
+        </is>
+      </c>
+      <c r="B823" s="15" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C823" s="15" t="inlineStr">
+        <is>
+          <t>La semana</t>
+        </is>
+      </c>
+      <c r="D823" s="15" t="inlineStr">
+        <is>
+          <t>Texto</t>
+        </is>
+      </c>
+      <c r="E823" s="15" t="inlineStr">
+        <is>
+          <t>Siempre</t>
+        </is>
+      </c>
+      <c r="F823" s="15" t="inlineStr">
+        <is>
+          <t>Grupo de otro curso: también cuenta para el máximo</t>
+        </is>
+      </c>
+      <c r="G823" s="13" t="inlineStr"/>
+      <c r="H823" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I823" s="13" t="inlineStr"/>
+      <c r="J823" s="15" t="inlineStr"/>
+      <c r="K823" s="16" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L823" s="16" t="inlineStr">
+        <is>
+          <t>Página (sitio/grupos.html)</t>
+        </is>
+      </c>
+    </row>
+    <row r="824">
+      <c r="A824" s="12" t="inlineStr">
+        <is>
+          <t>T823</t>
+        </is>
+      </c>
+      <c r="B824" s="12" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C824" s="12" t="inlineStr">
+        <is>
+          <t>La semana</t>
+        </is>
+      </c>
+      <c r="D824" s="12" t="inlineStr">
+        <is>
+          <t>Texto</t>
+        </is>
+      </c>
+      <c r="E824" s="12" t="inlineStr">
+        <is>
+          <t>Siempre</t>
+        </is>
+      </c>
+      <c r="F824" s="12" t="inlineStr">
+        <is>
+          <t>No disponible: ya pasó, faltan menos de 7 días o ya hay 2 grupos</t>
+        </is>
+      </c>
+      <c r="G824" s="13" t="inlineStr"/>
+      <c r="H824" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I824" s="13" t="inlineStr"/>
+      <c r="J824" s="12" t="inlineStr"/>
+      <c r="K824" s="14" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L824" s="14" t="inlineStr">
+        <is>
+          <t>Página (sitio/grupos.html)</t>
+        </is>
+      </c>
+    </row>
+    <row r="825">
+      <c r="A825" s="15" t="inlineStr">
+        <is>
+          <t>T824</t>
+        </is>
+      </c>
+      <c r="B825" s="15" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C825" s="15" t="inlineStr">
+        <is>
+          <t>La semana</t>
+        </is>
+      </c>
+      <c r="D825" s="15" t="inlineStr">
+        <is>
+          <t>Texto</t>
+        </is>
+      </c>
+      <c r="E825" s="15" t="inlineStr">
+        <is>
+          <t>Siempre</t>
+        </is>
+      </c>
+      <c r="F825" s="15" t="inlineStr">
+        <is>
+          <t>Sábado y domingo: no hay curso</t>
+        </is>
+      </c>
+      <c r="G825" s="13" t="inlineStr"/>
+      <c r="H825" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I825" s="13" t="inlineStr"/>
+      <c r="J825" s="15" t="inlineStr"/>
+      <c r="K825" s="16" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L825" s="16" t="inlineStr">
+        <is>
+          <t>Página (sitio/grupos.html)</t>
+        </is>
+      </c>
+    </row>
+    <row r="826">
+      <c r="A826" s="12" t="inlineStr">
+        <is>
+          <t>T825</t>
+        </is>
+      </c>
+      <c r="B826" s="12" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C826" s="12" t="inlineStr">
+        <is>
+          <t>La semana</t>
+        </is>
+      </c>
+      <c r="D826" s="12" t="inlineStr">
+        <is>
+          <t>Texto</t>
+        </is>
+      </c>
+      <c r="E826" s="12" t="inlineStr">
+        <is>
+          <t>Siempre</t>
+        </is>
+      </c>
+      <c r="F826" s="12" t="inlineStr">
+        <is>
+          <t>Día inhábil [por confirmar con el calendario oficial de la Secretaría]</t>
+        </is>
+      </c>
+      <c r="G826" s="13" t="inlineStr"/>
+      <c r="H826" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I826" s="13" t="inlineStr"/>
+      <c r="J826" s="12" t="inlineStr"/>
+      <c r="K826" s="14" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L826" s="14" t="inlineStr">
+        <is>
+          <t>Página (sitio/grupos.html)</t>
+        </is>
+      </c>
+    </row>
+    <row r="827">
+      <c r="A827" s="15" t="inlineStr">
+        <is>
+          <t>T826</t>
+        </is>
+      </c>
+      <c r="B827" s="15" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C827" s="15" t="inlineStr">
+        <is>
+          <t>La semana</t>
+        </is>
+      </c>
+      <c r="D827" s="15" t="inlineStr">
+        <is>
+          <t>Botón o enlace</t>
+        </is>
+      </c>
+      <c r="E827" s="15" t="inlineStr">
+        <is>
+          <t>Siempre</t>
+        </is>
+      </c>
+      <c r="F827" s="15" t="inlineStr">
+        <is>
+          <t>Atrás</t>
+        </is>
+      </c>
+      <c r="G827" s="13" t="inlineStr"/>
+      <c r="H827" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I827" s="13" t="inlineStr"/>
+      <c r="J827" s="15" t="inlineStr"/>
+      <c r="K827" s="16" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L827" s="16" t="inlineStr">
+        <is>
+          <t>Página (sitio/grupos.html)</t>
+        </is>
+      </c>
+    </row>
+    <row r="828">
+      <c r="A828" s="12" t="inlineStr">
+        <is>
+          <t>T827</t>
+        </is>
+      </c>
+      <c r="B828" s="12" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C828" s="12" t="inlineStr">
+        <is>
+          <t>La semana</t>
+        </is>
+      </c>
+      <c r="D828" s="12" t="inlineStr">
+        <is>
+          <t>Botón o enlace</t>
+        </is>
+      </c>
+      <c r="E828" s="12" t="inlineStr">
+        <is>
+          <t>Siempre</t>
+        </is>
+      </c>
+      <c r="F828" s="12" t="inlineStr">
+        <is>
+          <t>Siguiente</t>
+        </is>
+      </c>
+      <c r="G828" s="13" t="inlineStr"/>
+      <c r="H828" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I828" s="13" t="inlineStr"/>
+      <c r="J828" s="12" t="inlineStr"/>
+      <c r="K828" s="14" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L828" s="14" t="inlineStr">
+        <is>
+          <t>Página (sitio/grupos.html)</t>
+        </is>
+      </c>
+    </row>
+    <row r="829">
+      <c r="A829" s="15" t="inlineStr">
+        <is>
+          <t>T828</t>
+        </is>
+      </c>
+      <c r="B829" s="15" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C829" s="15" t="inlineStr">
+        <is>
+          <t>Quiénes van</t>
+        </is>
+      </c>
+      <c r="D829" s="15" t="inlineStr">
+        <is>
+          <t>Subtítulo</t>
+        </is>
+      </c>
+      <c r="E829" s="15" t="inlineStr">
+        <is>
+          <t>Siempre</t>
+        </is>
+      </c>
+      <c r="F829" s="15" t="inlineStr">
+        <is>
+          <t>¿Quiénes van?</t>
+        </is>
+      </c>
+      <c r="G829" s="13" t="inlineStr"/>
+      <c r="H829" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I829" s="13" t="inlineStr"/>
+      <c r="J829" s="15" t="inlineStr"/>
+      <c r="K829" s="16" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L829" s="16" t="inlineStr">
+        <is>
+          <t>Página (sitio/grupos.html)</t>
+        </is>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" s="12" t="inlineStr">
+        <is>
+          <t>T829</t>
+        </is>
+      </c>
+      <c r="B830" s="12" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C830" s="12" t="inlineStr">
+        <is>
+          <t>Quiénes van</t>
+        </is>
+      </c>
+      <c r="D830" s="12" t="inlineStr">
+        <is>
+          <t>Ayuda</t>
+        </is>
+      </c>
+      <c r="E830" s="12" t="inlineStr">
+        <is>
+          <t>Siempre</t>
+        </is>
+      </c>
+      <c r="F830" s="12" t="inlineStr">
+        <is>
+          <t>Si hay más de 25, entran las que más esperan y las de una misma institución de gobierno van juntas; el resto sigue en espera para otra semana.</t>
+        </is>
+      </c>
+      <c r="G830" s="13" t="inlineStr"/>
+      <c r="H830" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I830" s="13" t="inlineStr"/>
+      <c r="J830" s="12" t="inlineStr"/>
+      <c r="K830" s="14" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L830" s="14" t="inlineStr">
+        <is>
+          <t>Página (sitio/grupos.html)</t>
+        </is>
+      </c>
+    </row>
+    <row r="831">
+      <c r="A831" s="15" t="inlineStr">
+        <is>
+          <t>T830</t>
+        </is>
+      </c>
+      <c r="B831" s="15" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C831" s="15" t="inlineStr">
+        <is>
+          <t>Quiénes van</t>
+        </is>
+      </c>
+      <c r="D831" s="15" t="inlineStr">
+        <is>
+          <t>Pregunta</t>
+        </is>
+      </c>
+      <c r="E831" s="15" t="inlineStr">
+        <is>
+          <t>Siempre</t>
+        </is>
+      </c>
+      <c r="F831" s="15" t="inlineStr">
+        <is>
+          <t>¿De quiénes es el grupo?</t>
+        </is>
+      </c>
+      <c r="G831" s="13" t="inlineStr"/>
+      <c r="H831" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I831" s="13" t="inlineStr"/>
+      <c r="J831" s="15" t="inlineStr"/>
+      <c r="K831" s="16" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L831" s="16" t="inlineStr">
+        <is>
+          <t>Página (sitio/grupos.html)</t>
+        </is>
+      </c>
+    </row>
+    <row r="832">
+      <c r="A832" s="12" t="inlineStr">
+        <is>
+          <t>T831</t>
+        </is>
+      </c>
+      <c r="B832" s="12" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C832" s="12" t="inlineStr">
+        <is>
+          <t>Quiénes van</t>
+        </is>
+      </c>
+      <c r="D832" s="12" t="inlineStr">
+        <is>
+          <t>Opción</t>
+        </is>
+      </c>
+      <c r="E832" s="12" t="inlineStr">
+        <is>
+          <t>Siempre</t>
+        </is>
+      </c>
+      <c r="F832" s="12" t="inlineStr">
+        <is>
+          <t>Combinado — Recibe personas de cualquier organización e independientes.</t>
+        </is>
+      </c>
+      <c r="G832" s="13" t="inlineStr"/>
+      <c r="H832" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I832" s="13" t="inlineStr"/>
+      <c r="J832" s="12" t="inlineStr"/>
+      <c r="K832" s="14" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L832" s="14" t="inlineStr">
+        <is>
+          <t>Página (sitio/grupos.html)</t>
+        </is>
+      </c>
+    </row>
+    <row r="833">
+      <c r="A833" s="15" t="inlineStr">
+        <is>
+          <t>T832</t>
+        </is>
+      </c>
+      <c r="B833" s="15" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C833" s="15" t="inlineStr">
+        <is>
+          <t>Quiénes van</t>
+        </is>
+      </c>
+      <c r="D833" s="15" t="inlineStr">
+        <is>
+          <t>Opción</t>
+        </is>
+      </c>
+      <c r="E833" s="15" t="inlineStr">
+        <is>
+          <t>Siempre</t>
+        </is>
+      </c>
+      <c r="F833" s="15" t="inlineStr">
+        <is>
+          <t>Sólo de una organización — Recibe únicamente a la gente de esa organización: todas las elegidas tienen que ser de ella.</t>
+        </is>
+      </c>
+      <c r="G833" s="13" t="inlineStr"/>
+      <c r="H833" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I833" s="13" t="inlineStr"/>
+      <c r="J833" s="15" t="inlineStr"/>
+      <c r="K833" s="16" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L833" s="16" t="inlineStr">
+        <is>
+          <t>Página (sitio/grupos.html)</t>
+        </is>
+      </c>
+    </row>
+    <row r="834">
+      <c r="A834" s="12" t="inlineStr">
+        <is>
+          <t>T833</t>
+        </is>
+      </c>
+      <c r="B834" s="12" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C834" s="12" t="inlineStr">
+        <is>
+          <t>Quiénes van</t>
+        </is>
+      </c>
+      <c r="D834" s="12" t="inlineStr">
+        <is>
+          <t>Botón o enlace</t>
+        </is>
+      </c>
+      <c r="E834" s="12" t="inlineStr">
+        <is>
+          <t>Siempre</t>
+        </is>
+      </c>
+      <c r="F834" s="12" t="inlineStr">
+        <is>
+          <t>Atrás</t>
+        </is>
+      </c>
+      <c r="G834" s="13" t="inlineStr"/>
+      <c r="H834" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I834" s="13" t="inlineStr"/>
+      <c r="J834" s="12" t="inlineStr"/>
+      <c r="K834" s="14" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L834" s="14" t="inlineStr">
+        <is>
+          <t>Página (sitio/grupos.html)</t>
+        </is>
+      </c>
+    </row>
+    <row r="835">
+      <c r="A835" s="15" t="inlineStr">
+        <is>
+          <t>T834</t>
+        </is>
+      </c>
+      <c r="B835" s="15" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C835" s="15" t="inlineStr">
+        <is>
+          <t>Quiénes van</t>
+        </is>
+      </c>
+      <c r="D835" s="15" t="inlineStr">
+        <is>
+          <t>Botón o enlace</t>
+        </is>
+      </c>
+      <c r="E835" s="15" t="inlineStr">
+        <is>
+          <t>Siempre</t>
+        </is>
+      </c>
+      <c r="F835" s="15" t="inlineStr">
+        <is>
+          <t>Siguiente</t>
+        </is>
+      </c>
+      <c r="G835" s="13" t="inlineStr"/>
+      <c r="H835" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I835" s="13" t="inlineStr"/>
+      <c r="J835" s="15" t="inlineStr"/>
+      <c r="K835" s="16" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L835" s="16" t="inlineStr">
+        <is>
+          <t>Página (sitio/grupos.html)</t>
+        </is>
+      </c>
+    </row>
+    <row r="836">
+      <c r="A836" s="12" t="inlineStr">
+        <is>
+          <t>T835</t>
+        </is>
+      </c>
+      <c r="B836" s="12" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C836" s="12" t="inlineStr">
+        <is>
+          <t>Confirmar</t>
+        </is>
+      </c>
+      <c r="D836" s="12" t="inlineStr">
+        <is>
+          <t>Subtítulo</t>
+        </is>
+      </c>
+      <c r="E836" s="12" t="inlineStr">
+        <is>
+          <t>Siempre</t>
+        </is>
+      </c>
+      <c r="F836" s="12" t="inlineStr">
+        <is>
+          <t>Revise y confirme</t>
+        </is>
+      </c>
+      <c r="G836" s="13" t="inlineStr"/>
+      <c r="H836" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I836" s="13" t="inlineStr"/>
+      <c r="J836" s="12" t="inlineStr"/>
+      <c r="K836" s="14" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L836" s="14" t="inlineStr">
+        <is>
+          <t>Página (sitio/grupos.html)</t>
+        </is>
+      </c>
+    </row>
+    <row r="837">
+      <c r="A837" s="15" t="inlineStr">
+        <is>
+          <t>T836</t>
+        </is>
+      </c>
+      <c r="B837" s="15" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C837" s="15" t="inlineStr">
+        <is>
+          <t>Confirmar</t>
+        </is>
+      </c>
+      <c r="D837" s="15" t="inlineStr">
+        <is>
+          <t>Pregunta</t>
+        </is>
+      </c>
+      <c r="E837" s="15" t="inlineStr">
+        <is>
+          <t>Siempre</t>
+        </is>
+      </c>
+      <c r="F837" s="15" t="inlineStr">
+        <is>
+          <t>Instructor</t>
+        </is>
+      </c>
+      <c r="G837" s="13" t="inlineStr"/>
+      <c r="H837" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I837" s="13" t="inlineStr"/>
+      <c r="J837" s="15" t="inlineStr"/>
+      <c r="K837" s="16" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L837" s="16" t="inlineStr">
+        <is>
+          <t>Página (sitio/grupos.html)</t>
+        </is>
+      </c>
+    </row>
+    <row r="838">
+      <c r="A838" s="12" t="inlineStr">
+        <is>
+          <t>T837</t>
+        </is>
+      </c>
+      <c r="B838" s="12" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C838" s="12" t="inlineStr">
+        <is>
+          <t>Confirmar</t>
+        </is>
+      </c>
+      <c r="D838" s="12" t="inlineStr">
+        <is>
+          <t>Ayuda</t>
+        </is>
+      </c>
+      <c r="E838" s="12" t="inlineStr">
+        <is>
+          <t>Siempre</t>
+        </is>
+      </c>
+      <c r="F838" s="12" t="inlineStr">
+        <is>
+          <t>Se indica si ya tiene otro curso esas fechas.</t>
+        </is>
+      </c>
+      <c r="G838" s="13" t="inlineStr"/>
+      <c r="H838" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I838" s="13" t="inlineStr"/>
+      <c r="J838" s="12" t="inlineStr"/>
+      <c r="K838" s="14" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L838" s="14" t="inlineStr">
+        <is>
+          <t>Página (sitio/grupos.html)</t>
+        </is>
+      </c>
+    </row>
+    <row r="839">
+      <c r="A839" s="15" t="inlineStr">
+        <is>
+          <t>T838</t>
+        </is>
+      </c>
+      <c r="B839" s="15" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C839" s="15" t="inlineStr">
+        <is>
+          <t>Confirmar</t>
+        </is>
+      </c>
+      <c r="D839" s="15" t="inlineStr">
+        <is>
+          <t>Indicación de lista</t>
+        </is>
+      </c>
+      <c r="E839" s="15" t="inlineStr">
+        <is>
+          <t>Siempre</t>
+        </is>
+      </c>
+      <c r="F839" s="15" t="inlineStr">
+        <is>
+          <t>Por asignar</t>
+        </is>
+      </c>
+      <c r="G839" s="13" t="inlineStr"/>
+      <c r="H839" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I839" s="13" t="inlineStr"/>
+      <c r="J839" s="15" t="inlineStr"/>
+      <c r="K839" s="16" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L839" s="16" t="inlineStr">
+        <is>
+          <t>Página (sitio/grupos.html)</t>
+        </is>
+      </c>
+    </row>
+    <row r="840">
+      <c r="A840" s="12" t="inlineStr">
+        <is>
+          <t>T839</t>
+        </is>
+      </c>
+      <c r="B840" s="12" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C840" s="12" t="inlineStr">
+        <is>
+          <t>Confirmar</t>
+        </is>
+      </c>
+      <c r="D840" s="12" t="inlineStr">
+        <is>
+          <t>Opción de lista</t>
+        </is>
+      </c>
+      <c r="E840" s="12" t="inlineStr">
+        <is>
+          <t>Siempre</t>
+        </is>
+      </c>
+      <c r="F840" s="12" t="inlineStr">
+        <is>
+          <t>Laura Ejemplo Instructora</t>
+        </is>
+      </c>
+      <c r="G840" s="13" t="inlineStr"/>
+      <c r="H840" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I840" s="13" t="inlineStr"/>
+      <c r="J840" s="12" t="inlineStr"/>
+      <c r="K840" s="14" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L840" s="14" t="inlineStr">
+        <is>
+          <t>Página (sitio/grupos.html)</t>
+        </is>
+      </c>
+    </row>
+    <row r="841">
+      <c r="A841" s="15" t="inlineStr">
+        <is>
+          <t>T840</t>
+        </is>
+      </c>
+      <c r="B841" s="15" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C841" s="15" t="inlineStr">
+        <is>
+          <t>Confirmar</t>
+        </is>
+      </c>
+      <c r="D841" s="15" t="inlineStr">
+        <is>
+          <t>Opción de lista</t>
+        </is>
+      </c>
+      <c r="E841" s="15" t="inlineStr">
+        <is>
+          <t>Siempre</t>
+        </is>
+      </c>
+      <c r="F841" s="15" t="inlineStr">
+        <is>
+          <t>Instructor Ejemplo Dos</t>
+        </is>
+      </c>
+      <c r="G841" s="13" t="inlineStr"/>
+      <c r="H841" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I841" s="13" t="inlineStr"/>
+      <c r="J841" s="15" t="inlineStr"/>
+      <c r="K841" s="16" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L841" s="16" t="inlineStr">
+        <is>
+          <t>Página (sitio/grupos.html)</t>
+        </is>
+      </c>
+    </row>
+    <row r="842">
+      <c r="A842" s="12" t="inlineStr">
+        <is>
+          <t>T841</t>
+        </is>
+      </c>
+      <c r="B842" s="12" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C842" s="12" t="inlineStr">
+        <is>
+          <t>Confirmar</t>
+        </is>
+      </c>
+      <c r="D842" s="12" t="inlineStr">
+        <is>
+          <t>Pregunta</t>
+        </is>
+      </c>
+      <c r="E842" s="12" t="inlineStr">
+        <is>
+          <t>Siempre</t>
+        </is>
+      </c>
+      <c r="F842" s="12" t="inlineStr">
+        <is>
+          <t>Hora de entrada</t>
+        </is>
+      </c>
+      <c r="G842" s="13" t="inlineStr"/>
+      <c r="H842" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I842" s="13" t="inlineStr"/>
+      <c r="J842" s="12" t="inlineStr"/>
+      <c r="K842" s="14" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L842" s="14" t="inlineStr">
+        <is>
+          <t>Página (sitio/grupos.html)</t>
+        </is>
+      </c>
+    </row>
+    <row r="843">
+      <c r="A843" s="15" t="inlineStr">
+        <is>
+          <t>T842</t>
+        </is>
+      </c>
+      <c r="B843" s="15" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C843" s="15" t="inlineStr">
+        <is>
+          <t>Confirmar</t>
+        </is>
+      </c>
+      <c r="D843" s="15" t="inlineStr">
+        <is>
+          <t>Ayuda</t>
+        </is>
+      </c>
+      <c r="E843" s="15" t="inlineStr">
+        <is>
+          <t>Siempre</t>
+        </is>
+      </c>
+      <c r="F843" s="15" t="inlineStr">
+        <is>
+          <t>El curso es de 9:00 a 15:00 todos sus días.</t>
+        </is>
+      </c>
+      <c r="G843" s="13" t="inlineStr"/>
+      <c r="H843" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I843" s="13" t="inlineStr"/>
+      <c r="J843" s="15" t="inlineStr"/>
+      <c r="K843" s="16" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L843" s="16" t="inlineStr">
+        <is>
+          <t>Página (sitio/grupos.html)</t>
+        </is>
+      </c>
+    </row>
+    <row r="844">
+      <c r="A844" s="12" t="inlineStr">
+        <is>
+          <t>T843</t>
+        </is>
+      </c>
+      <c r="B844" s="12" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C844" s="12" t="inlineStr">
+        <is>
+          <t>Confirmar</t>
+        </is>
+      </c>
+      <c r="D844" s="12" t="inlineStr">
+        <is>
+          <t>Indicación de lista</t>
+        </is>
+      </c>
+      <c r="E844" s="12" t="inlineStr">
+        <is>
+          <t>Siempre</t>
+        </is>
+      </c>
+      <c r="F844" s="12" t="inlineStr">
+        <is>
+          <t>Elija</t>
+        </is>
+      </c>
+      <c r="G844" s="13" t="inlineStr"/>
+      <c r="H844" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I844" s="13" t="inlineStr"/>
+      <c r="J844" s="12" t="inlineStr"/>
+      <c r="K844" s="14" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L844" s="14" t="inlineStr">
+        <is>
+          <t>Página (sitio/grupos.html)</t>
+        </is>
+      </c>
+    </row>
+    <row r="845">
+      <c r="A845" s="15" t="inlineStr">
+        <is>
+          <t>T844</t>
+        </is>
+      </c>
+      <c r="B845" s="15" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C845" s="15" t="inlineStr">
+        <is>
+          <t>Confirmar</t>
+        </is>
+      </c>
+      <c r="D845" s="15" t="inlineStr">
+        <is>
+          <t>Botón o enlace</t>
+        </is>
+      </c>
+      <c r="E845" s="15" t="inlineStr">
+        <is>
+          <t>Siempre</t>
+        </is>
+      </c>
+      <c r="F845" s="15" t="inlineStr">
+        <is>
+          <t>Atrás</t>
+        </is>
+      </c>
+      <c r="G845" s="13" t="inlineStr"/>
+      <c r="H845" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I845" s="13" t="inlineStr"/>
+      <c r="J845" s="15" t="inlineStr"/>
+      <c r="K845" s="16" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L845" s="16" t="inlineStr">
+        <is>
+          <t>Página (sitio/grupos.html)</t>
+        </is>
+      </c>
+    </row>
+    <row r="846">
+      <c r="A846" s="12" t="inlineStr">
+        <is>
+          <t>T845</t>
+        </is>
+      </c>
+      <c r="B846" s="12" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C846" s="12" t="inlineStr">
+        <is>
+          <t>Confirmar</t>
+        </is>
+      </c>
+      <c r="D846" s="12" t="inlineStr">
+        <is>
+          <t>Botón o enlace</t>
+        </is>
+      </c>
+      <c r="E846" s="12" t="inlineStr">
+        <is>
+          <t>Siempre</t>
+        </is>
+      </c>
+      <c r="F846" s="12" t="inlineStr">
+        <is>
+          <t>Crear sin confirmar</t>
+        </is>
+      </c>
+      <c r="G846" s="13" t="inlineStr"/>
+      <c r="H846" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I846" s="13" t="inlineStr"/>
+      <c r="J846" s="12" t="inlineStr"/>
+      <c r="K846" s="14" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L846" s="14" t="inlineStr">
+        <is>
+          <t>Página (sitio/grupos.html)</t>
+        </is>
+      </c>
+    </row>
+    <row r="847">
+      <c r="A847" s="15" t="inlineStr">
+        <is>
+          <t>T846</t>
+        </is>
+      </c>
+      <c r="B847" s="15" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C847" s="15" t="inlineStr">
+        <is>
+          <t>Confirmar</t>
+        </is>
+      </c>
+      <c r="D847" s="15" t="inlineStr">
+        <is>
+          <t>Botón o enlace</t>
+        </is>
+      </c>
+      <c r="E847" s="15" t="inlineStr">
+        <is>
+          <t>Siempre</t>
+        </is>
+      </c>
+      <c r="F847" s="15" t="inlineStr">
+        <is>
+          <t>Crear el grupo</t>
+        </is>
+      </c>
+      <c r="G847" s="13" t="inlineStr"/>
+      <c r="H847" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I847" s="13" t="inlineStr"/>
+      <c r="J847" s="15" t="inlineStr"/>
+      <c r="K847" s="16" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L847" s="16" t="inlineStr">
+        <is>
+          <t>Página (sitio/grupos.html)</t>
+        </is>
+      </c>
+    </row>
+    <row r="848">
+      <c r="A848" s="12" t="inlineStr">
+        <is>
+          <t>T847</t>
+        </is>
+      </c>
+      <c r="B848" s="12" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C848" s="12" t="inlineStr">
+        <is>
+          <t>Grupos programados</t>
+        </is>
+      </c>
+      <c r="D848" s="12" t="inlineStr">
+        <is>
+          <t>Subtítulo</t>
+        </is>
+      </c>
+      <c r="E848" s="12" t="inlineStr">
+        <is>
+          <t>Siempre</t>
+        </is>
+      </c>
+      <c r="F848" s="12" t="inlineStr">
+        <is>
+          <t>Grupos programados</t>
+        </is>
+      </c>
+      <c r="G848" s="13" t="inlineStr"/>
+      <c r="H848" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I848" s="13" t="inlineStr"/>
+      <c r="J848" s="12" t="inlineStr"/>
+      <c r="K848" s="14" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L848" s="14" t="inlineStr">
+        <is>
+          <t>Página (sitio/grupos.html)</t>
+        </is>
+      </c>
+    </row>
+    <row r="849">
+      <c r="A849" s="15" t="inlineStr">
+        <is>
+          <t>T848</t>
+        </is>
+      </c>
+      <c r="B849" s="15" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C849" s="15" t="inlineStr">
+        <is>
+          <t>Grupos programados</t>
+        </is>
+      </c>
+      <c r="D849" s="15" t="inlineStr">
+        <is>
+          <t>Introducción</t>
+        </is>
+      </c>
+      <c r="E849" s="15" t="inlineStr">
+        <is>
+          <t>Siempre</t>
+        </is>
+      </c>
+      <c r="F849" s="15" t="inlineStr">
+        <is>
+          <t>Por curso: los grupos por confirmar, confirmados y en curso, con lo que les falta.</t>
+        </is>
+      </c>
+      <c r="G849" s="13" t="inlineStr"/>
+      <c r="H849" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I849" s="13" t="inlineStr"/>
+      <c r="J849" s="15" t="inlineStr"/>
+      <c r="K849" s="16" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L849" s="16" t="inlineStr">
+        <is>
+          <t>Página (sitio/grupos.html)</t>
+        </is>
+      </c>
+    </row>
+    <row r="850">
+      <c r="A850" s="12" t="inlineStr">
+        <is>
+          <t>T849</t>
+        </is>
+      </c>
+      <c r="B850" s="12" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C850" s="12" t="inlineStr">
+        <is>
+          <t>Grupos programados</t>
+        </is>
+      </c>
+      <c r="D850" s="12" t="inlineStr">
+        <is>
+          <t>Título desplegable</t>
+        </is>
+      </c>
+      <c r="E850" s="12" t="inlineStr">
+        <is>
+          <t>Siempre</t>
+        </is>
+      </c>
+      <c r="F850" s="12" t="inlineStr">
+        <is>
+          <t>Grupos que ya terminaron</t>
+        </is>
+      </c>
+      <c r="G850" s="13" t="inlineStr"/>
+      <c r="H850" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I850" s="13" t="inlineStr"/>
+      <c r="J850" s="12" t="inlineStr"/>
+      <c r="K850" s="14" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L850" s="14" t="inlineStr">
+        <is>
+          <t>Página (sitio/grupos.html)</t>
+        </is>
+      </c>
+    </row>
+    <row r="851">
+      <c r="A851" s="15" t="inlineStr">
+        <is>
+          <t>T850</t>
+        </is>
+      </c>
+      <c r="B851" s="15" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C851" s="15" t="inlineStr">
+        <is>
+          <t>Grupos programados</t>
+        </is>
+      </c>
+      <c r="D851" s="15" t="inlineStr">
+        <is>
+          <t>Ayuda</t>
+        </is>
+      </c>
+      <c r="E851" s="15" t="inlineStr">
+        <is>
+          <t>Siempre</t>
+        </is>
+      </c>
+      <c r="F851" s="15" t="inlineStr">
+        <is>
+          <t>Los cuatro cursos nunca se mezclan; un grupo se confirma con al menos 5 personas, hora de entrada e instructor, y recibe hasta 25. Pendiente (P92): quién arma los grupos (hoy, el perfil de revisión y cotejo) y quién asigna a los instructores.</t>
+        </is>
+      </c>
+      <c r="G851" s="13" t="inlineStr"/>
+      <c r="H851" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I851" s="13" t="inlineStr"/>
+      <c r="J851" s="15" t="inlineStr"/>
+      <c r="K851" s="16" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L851" s="16" t="inlineStr">
+        <is>
+          <t>Página (sitio/grupos.html)</t>
+        </is>
+      </c>
+    </row>
+    <row r="852">
+      <c r="A852" s="12" t="inlineStr">
+        <is>
+          <t>T851</t>
+        </is>
+      </c>
+      <c r="B852" s="12" t="inlineStr">
+        <is>
+          <t>Reposición de tu credencial</t>
+        </is>
+      </c>
+      <c r="C852" s="12" t="inlineStr">
+        <is>
+          <t>Resultado</t>
+        </is>
+      </c>
+      <c r="D852" s="12" t="inlineStr">
+        <is>
+          <t>Título</t>
+        </is>
+      </c>
+      <c r="E852" s="12" t="inlineStr">
+        <is>
+          <t>Al pedirla o al cargar el acta corregida</t>
+        </is>
+      </c>
+      <c r="F852" s="12" t="inlineStr">
+        <is>
+          <t>Recibimos tu solicitud de reposición · Recibimos tu acta corregida</t>
+        </is>
+      </c>
+      <c r="G852" s="13" t="inlineStr"/>
+      <c r="H852" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I852" s="13" t="inlineStr"/>
+      <c r="J852" s="12" t="inlineStr"/>
+      <c r="K852" s="14" t="inlineStr">
+        <is>
+          <t>Persona solicitante</t>
+        </is>
+      </c>
+      <c r="L852" s="14" t="inlineStr">
+        <is>
           <t>Código del sitio (sitio/app/reposicion.js)</t>
         </is>
       </c>
     </row>
+    <row r="853">
+      <c r="A853" s="15" t="inlineStr">
+        <is>
+          <t>T852</t>
+        </is>
+      </c>
+      <c r="B853" s="15" t="inlineStr">
+        <is>
+          <t>Reposición de tu credencial</t>
+        </is>
+      </c>
+      <c r="C853" s="15" t="inlineStr">
+        <is>
+          <t>Resultado</t>
+        </is>
+      </c>
+      <c r="D853" s="15" t="inlineStr">
+        <is>
+          <t>Pasos</t>
+        </is>
+      </c>
+      <c r="E853" s="15" t="inlineStr">
+        <is>
+          <t>Al pedirla</t>
+        </is>
+      </c>
+      <c r="F853" s="15" t="inlineStr">
+        <is>
+          <t>La Secretaría revisa tu acta. · Te indica en «Mis trámites» si debes corregir algo o, si está completa, cuánto pagar. · Pagas la cuota de reposición y recoges tu credencial en la oficina del Vivero Nezahualcóyotl, con el mismo número y la misma vigencia.</t>
+        </is>
+      </c>
+      <c r="G853" s="13" t="inlineStr"/>
+      <c r="H853" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I853" s="13" t="inlineStr"/>
+      <c r="J853" s="15" t="inlineStr"/>
+      <c r="K853" s="16" t="inlineStr">
+        <is>
+          <t>Persona solicitante</t>
+        </is>
+      </c>
+      <c r="L853" s="16" t="inlineStr">
+        <is>
+          <t>Código del sitio (sitio/app/reposicion.js)</t>
+        </is>
+      </c>
+    </row>
+    <row r="854">
+      <c r="A854" s="12" t="inlineStr">
+        <is>
+          <t>T853</t>
+        </is>
+      </c>
+      <c r="B854" s="12" t="inlineStr">
+        <is>
+          <t>Reposición de tu credencial</t>
+        </is>
+      </c>
+      <c r="C854" s="12" t="inlineStr">
+        <is>
+          <t>Acreditación</t>
+        </is>
+      </c>
+      <c r="D854" s="12" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="E854" s="12" t="inlineStr">
+        <is>
+          <t>Credencial del sistema que todavía no se entrega</t>
+        </is>
+      </c>
+      <c r="F854" s="12" t="inlineStr">
+        <is>
+          <t>Tu credencial todavía no se te entrega: recógela en la oficina del Vivero. La reposición es para una credencial que ya recibiste y perdiste o te robaron.</t>
+        </is>
+      </c>
+      <c r="G854" s="13" t="inlineStr"/>
+      <c r="H854" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I854" s="13" t="inlineStr"/>
+      <c r="J854" s="12" t="inlineStr"/>
+      <c r="K854" s="14" t="inlineStr">
+        <is>
+          <t>Persona solicitante</t>
+        </is>
+      </c>
+      <c r="L854" s="14" t="inlineStr">
+        <is>
+          <t>Código del sitio (sitio/app/reposicion.js)</t>
+        </is>
+      </c>
+    </row>
+    <row r="855">
+      <c r="A855" s="15" t="inlineStr">
+        <is>
+          <t>T854</t>
+        </is>
+      </c>
+      <c r="B855" s="15" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C855" s="15" t="inlineStr">
+        <is>
+          <t>Cabecera</t>
+        </is>
+      </c>
+      <c r="D855" s="15" t="inlineStr">
+        <is>
+          <t>Texto</t>
+        </is>
+      </c>
+      <c r="E855" s="15" t="inlineStr">
+        <is>
+          <t>Siempre</t>
+        </is>
+      </c>
+      <c r="F855" s="15" t="inlineStr">
+        <is>
+          <t>Hoy es DÍA N de MES de AAAA. Arme un grupo en cuatro pasos: el curso, la semana, quiénes van y confirmar.</t>
+        </is>
+      </c>
+      <c r="G855" s="13" t="inlineStr"/>
+      <c r="H855" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I855" s="13" t="inlineStr"/>
+      <c r="J855" s="15" t="inlineStr"/>
+      <c r="K855" s="16" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L855" s="16" t="inlineStr">
+        <is>
+          <t>Código del sitio (sitio/app/grupos.js)</t>
+        </is>
+      </c>
+    </row>
+    <row r="856">
+      <c r="A856" s="12" t="inlineStr">
+        <is>
+          <t>T855</t>
+        </is>
+      </c>
+      <c r="B856" s="12" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C856" s="12" t="inlineStr">
+        <is>
+          <t>Paso 1 · el curso</t>
+        </is>
+      </c>
+      <c r="D856" s="12" t="inlineStr">
+        <is>
+          <t>Texto</t>
+        </is>
+      </c>
+      <c r="E856" s="12" t="inlineStr">
+        <is>
+          <t>En cada curso</t>
+        </is>
+      </c>
+      <c r="F856" s="12" t="inlineStr">
+        <is>
+          <t>N personas en espera · N esperan 15 días o más · N ya vencidas · Falta gente para un grupo (mínimo 5) / Alcanza para N grupos nuevos de hasta 25 / Nadie espera por ahora</t>
+        </is>
+      </c>
+      <c r="G856" s="13" t="inlineStr"/>
+      <c r="H856" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I856" s="13" t="inlineStr"/>
+      <c r="J856" s="12" t="inlineStr"/>
+      <c r="K856" s="14" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L856" s="14" t="inlineStr">
+        <is>
+          <t>Código del sitio (sitio/app/grupos.js)</t>
+        </is>
+      </c>
+    </row>
+    <row r="857">
+      <c r="A857" s="15" t="inlineStr">
+        <is>
+          <t>T856</t>
+        </is>
+      </c>
+      <c r="B857" s="15" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C857" s="15" t="inlineStr">
+        <is>
+          <t>Paso 2 · la semana</t>
+        </is>
+      </c>
+      <c r="D857" s="15" t="inlineStr">
+        <is>
+          <t>Texto</t>
+        </is>
+      </c>
+      <c r="E857" s="15" t="inlineStr">
+        <is>
+          <t>Siempre</t>
+        </is>
+      </c>
+      <c r="F857" s="15" t="inlineStr">
+        <is>
+          <t>CURSO · lunes a viernes, de 9:00 a 15:00 (o «un día, de 9:00 a 15:00»). Puede haber 2 grupos al mismo tiempo, de cualquier curso; el curso empieza al menos 7 días después de confirmarlo.</t>
+        </is>
+      </c>
+      <c r="G857" s="13" t="inlineStr"/>
+      <c r="H857" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I857" s="13" t="inlineStr"/>
+      <c r="J857" s="15" t="inlineStr"/>
+      <c r="K857" s="16" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L857" s="16" t="inlineStr">
+        <is>
+          <t>Código del sitio (sitio/app/grupos.js)</t>
+        </is>
+      </c>
+    </row>
+    <row r="858">
+      <c r="A858" s="12" t="inlineStr">
+        <is>
+          <t>T857</t>
+        </is>
+      </c>
+      <c r="B858" s="12" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C858" s="12" t="inlineStr">
+        <is>
+          <t>Paso 2 · columna «Semana»</t>
+        </is>
+      </c>
+      <c r="D858" s="12" t="inlineStr">
+        <is>
+          <t>Botón</t>
+        </is>
+      </c>
+      <c r="E858" s="12" t="inlineStr">
+        <is>
+          <t>Semana que se puede elegir</t>
+        </is>
+      </c>
+      <c r="F858" s="12" t="inlineStr">
+        <is>
+          <t>Libre · 2 lugares libres / 1 lugar libre de 2 (elegida: «Elegida»). Nombre para el lector: «Elegir la semana del 2 al 6 de noviembre de 2026: 2 lugares libres»</t>
+        </is>
+      </c>
+      <c r="G858" s="13" t="inlineStr"/>
+      <c r="H858" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I858" s="13" t="inlineStr"/>
+      <c r="J858" s="12" t="inlineStr"/>
+      <c r="K858" s="14" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L858" s="14" t="inlineStr">
+        <is>
+          <t>Código del sitio (sitio/app/grupos.js)</t>
+        </is>
+      </c>
+    </row>
+    <row r="859">
+      <c r="A859" s="15" t="inlineStr">
+        <is>
+          <t>T858</t>
+        </is>
+      </c>
+      <c r="B859" s="15" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C859" s="15" t="inlineStr">
+        <is>
+          <t>Paso 2 · columna «Semana»</t>
+        </is>
+      </c>
+      <c r="D859" s="15" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="E859" s="15" t="inlineStr">
+        <is>
+          <t>Semana que no se puede elegir</t>
+        </is>
+      </c>
+      <c r="F859" s="15" t="inlineStr">
+        <is>
+          <t>No disponible · Ya pasó / Ya empezó / Faltan menos de 7 días / Ya hay 2 grupos / Día inhábil / Falta más de un año</t>
+        </is>
+      </c>
+      <c r="G859" s="13" t="inlineStr"/>
+      <c r="H859" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I859" s="13" t="inlineStr"/>
+      <c r="J859" s="15" t="inlineStr"/>
+      <c r="K859" s="16" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L859" s="16" t="inlineStr">
+        <is>
+          <t>Código del sitio (sitio/app/grupos.js)</t>
+        </is>
+      </c>
+    </row>
+    <row r="860">
+      <c r="A860" s="12" t="inlineStr">
+        <is>
+          <t>T859</t>
+        </is>
+      </c>
+      <c r="B860" s="12" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C860" s="12" t="inlineStr">
+        <is>
+          <t>Paso 2 · calendario</t>
+        </is>
+      </c>
+      <c r="D860" s="12" t="inlineStr">
+        <is>
+          <t>Etiqueta</t>
+        </is>
+      </c>
+      <c r="E860" s="12" t="inlineStr">
+        <is>
+          <t>En los días</t>
+        </is>
+      </c>
+      <c r="F860" s="12" t="inlineStr">
+        <is>
+          <t>G-AAAA-NNN (folio, el primer día) · Examen (el último) · Nuevo grupo (la semana elegida) · Hoy · Inhábil</t>
+        </is>
+      </c>
+      <c r="G860" s="13" t="inlineStr"/>
+      <c r="H860" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I860" s="13" t="inlineStr"/>
+      <c r="J860" s="12" t="inlineStr"/>
+      <c r="K860" s="14" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L860" s="14" t="inlineStr">
+        <is>
+          <t>Código del sitio (sitio/app/grupos.js)</t>
+        </is>
+      </c>
+    </row>
+    <row r="861">
+      <c r="A861" s="15" t="inlineStr">
+        <is>
+          <t>T860</t>
+        </is>
+      </c>
+      <c r="B861" s="15" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C861" s="15" t="inlineStr">
+        <is>
+          <t>Paso 2 · semana elegida</t>
+        </is>
+      </c>
+      <c r="D861" s="15" t="inlineStr">
+        <is>
+          <t>Texto</t>
+        </is>
+      </c>
+      <c r="E861" s="15" t="inlineStr">
+        <is>
+          <t>Con una semana elegida</t>
+        </is>
+      </c>
+      <c r="F861" s="15" t="inlineStr">
+        <is>
+          <t>Del 2 al 6 de noviembre · Del lunes 2 de noviembre de 2026 al viernes 6 de noviembre de 2026, de 9:00 a 15:00. El viernes, repaso de conocimientos y examen final en el PILARES. (Curso de un día: «El DÍA…, de 9:00 a 15:00, con el examen ese mismo día en el PILARES».)</t>
+        </is>
+      </c>
+      <c r="G861" s="13" t="inlineStr"/>
+      <c r="H861" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I861" s="13" t="inlineStr"/>
+      <c r="J861" s="15" t="inlineStr"/>
+      <c r="K861" s="16" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L861" s="16" t="inlineStr">
+        <is>
+          <t>Código del sitio (sitio/app/grupos.js)</t>
+        </is>
+      </c>
+    </row>
+    <row r="862">
+      <c r="A862" s="12" t="inlineStr">
+        <is>
+          <t>T861</t>
+        </is>
+      </c>
+      <c r="B862" s="12" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C862" s="12" t="inlineStr">
+        <is>
+          <t>Paso 2 · semana elegida</t>
+        </is>
+      </c>
+      <c r="D862" s="12" t="inlineStr">
+        <is>
+          <t>Texto</t>
+        </is>
+      </c>
+      <c r="E862" s="12" t="inlineStr">
+        <is>
+          <t>Sin semana</t>
+        </is>
+      </c>
+      <c r="F862" s="12" t="inlineStr">
+        <is>
+          <t>Ninguna todavía · Toque «Libre» en la semana que quiere. (Grupo que ya existe: «Sin semana todavía · … o siga sin semana: el grupo la conserva como está».)</t>
+        </is>
+      </c>
+      <c r="G862" s="13" t="inlineStr"/>
+      <c r="H862" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I862" s="13" t="inlineStr"/>
+      <c r="J862" s="12" t="inlineStr"/>
+      <c r="K862" s="14" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L862" s="14" t="inlineStr">
+        <is>
+          <t>Código del sitio (sitio/app/grupos.js)</t>
+        </is>
+      </c>
+    </row>
+    <row r="863">
+      <c r="A863" s="15" t="inlineStr">
+        <is>
+          <t>T862</t>
+        </is>
+      </c>
+      <c r="B863" s="15" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C863" s="15" t="inlineStr">
+        <is>
+          <t>Paso 2</t>
+        </is>
+      </c>
+      <c r="D863" s="15" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="E863" s="15" t="inlineStr">
+        <is>
+          <t>Siguiente sin semana</t>
+        </is>
+      </c>
+      <c r="F863" s="15" t="inlineStr">
+        <is>
+          <t>Elija una semana libre en el calendario: toque «Libre» en la semana que quiere.</t>
+        </is>
+      </c>
+      <c r="G863" s="13" t="inlineStr"/>
+      <c r="H863" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I863" s="13" t="inlineStr"/>
+      <c r="J863" s="15" t="inlineStr"/>
+      <c r="K863" s="16" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L863" s="16" t="inlineStr">
+        <is>
+          <t>Código del sitio (sitio/app/grupos.js)</t>
+        </is>
+      </c>
+    </row>
+    <row r="864">
+      <c r="A864" s="12" t="inlineStr">
+        <is>
+          <t>T863</t>
+        </is>
+      </c>
+      <c r="B864" s="12" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C864" s="12" t="inlineStr">
+        <is>
+          <t>Paso 2</t>
+        </is>
+      </c>
+      <c r="D864" s="12" t="inlineStr">
+        <is>
+          <t>Aviso</t>
+        </is>
+      </c>
+      <c r="E864" s="12" t="inlineStr">
+        <is>
+          <t>Al tocar un día que no se puede</t>
+        </is>
+      </c>
+      <c r="F864" s="12" t="inlineStr">
+        <is>
+          <t>El DÍA no se puede: RAZÓN.</t>
+        </is>
+      </c>
+      <c r="G864" s="13" t="inlineStr"/>
+      <c r="H864" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I864" s="13" t="inlineStr"/>
+      <c r="J864" s="12" t="inlineStr"/>
+      <c r="K864" s="14" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L864" s="14" t="inlineStr">
+        <is>
+          <t>Código del sitio (sitio/app/grupos.js)</t>
+        </is>
+      </c>
+    </row>
+    <row r="865">
+      <c r="A865" s="15" t="inlineStr">
+        <is>
+          <t>T864</t>
+        </is>
+      </c>
+      <c r="B865" s="15" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C865" s="15" t="inlineStr">
+        <is>
+          <t>Paso 3 · quiénes van</t>
+        </is>
+      </c>
+      <c r="D865" s="15" t="inlineStr">
+        <is>
+          <t>Texto</t>
+        </is>
+      </c>
+      <c r="E865" s="15" t="inlineStr">
+        <is>
+          <t>Grupo nuevo</t>
+        </is>
+      </c>
+      <c r="F865" s="15" t="inlineStr">
+        <is>
+          <t>Se proponen las N personas que más esperan, primero las prioritarias y las de una misma institución de gobierno juntas. Quite o agregue a quien haga falta.</t>
+        </is>
+      </c>
+      <c r="G865" s="13" t="inlineStr"/>
+      <c r="H865" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I865" s="13" t="inlineStr"/>
+      <c r="J865" s="15" t="inlineStr"/>
+      <c r="K865" s="16" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L865" s="16" t="inlineStr">
+        <is>
+          <t>Código del sitio (sitio/app/grupos.js)</t>
+        </is>
+      </c>
+    </row>
+    <row r="866">
+      <c r="A866" s="12" t="inlineStr">
+        <is>
+          <t>T865</t>
+        </is>
+      </c>
+      <c r="B866" s="12" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C866" s="12" t="inlineStr">
+        <is>
+          <t>Paso 3 · quiénes van</t>
+        </is>
+      </c>
+      <c r="D866" s="12" t="inlineStr">
+        <is>
+          <t>Texto</t>
+        </is>
+      </c>
+      <c r="E866" s="12" t="inlineStr">
+        <is>
+          <t>Siempre</t>
+        </is>
+      </c>
+      <c r="F866" s="12" t="inlineStr">
+        <is>
+          <t>N de 25 lugares · se confirma con al menos 5 personas</t>
+        </is>
+      </c>
+      <c r="G866" s="13" t="inlineStr"/>
+      <c r="H866" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I866" s="13" t="inlineStr"/>
+      <c r="J866" s="12" t="inlineStr"/>
+      <c r="K866" s="14" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L866" s="14" t="inlineStr">
+        <is>
+          <t>Código del sitio (sitio/app/grupos.js)</t>
+        </is>
+      </c>
+    </row>
+    <row r="867">
+      <c r="A867" s="15" t="inlineStr">
+        <is>
+          <t>T866</t>
+        </is>
+      </c>
+      <c r="B867" s="15" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C867" s="15" t="inlineStr">
+        <is>
+          <t>Paso 3 · quiénes van</t>
+        </is>
+      </c>
+      <c r="D867" s="15" t="inlineStr">
+        <is>
+          <t>Plegable</t>
+        </is>
+      </c>
+      <c r="E867" s="15" t="inlineStr">
+        <is>
+          <t>Con más en espera que las propuestas</t>
+        </is>
+      </c>
+      <c r="F867" s="15" t="inlineStr">
+        <is>
+          <t>Cambiar a quiénes van (N más en espera)</t>
+        </is>
+      </c>
+      <c r="G867" s="13" t="inlineStr"/>
+      <c r="H867" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I867" s="13" t="inlineStr"/>
+      <c r="J867" s="15" t="inlineStr"/>
+      <c r="K867" s="16" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L867" s="16" t="inlineStr">
+        <is>
+          <t>Código del sitio (sitio/app/grupos.js)</t>
+        </is>
+      </c>
+    </row>
+    <row r="868">
+      <c r="A868" s="12" t="inlineStr">
+        <is>
+          <t>T867</t>
+        </is>
+      </c>
+      <c r="B868" s="12" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C868" s="12" t="inlineStr">
+        <is>
+          <t>Paso 3</t>
+        </is>
+      </c>
+      <c r="D868" s="12" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="E868" s="12" t="inlineStr">
+        <is>
+          <t>Siguiente sin nadie</t>
+        </is>
+      </c>
+      <c r="F868" s="12" t="inlineStr">
+        <is>
+          <t>Elija a quién va · Marque la casilla junto al nombre de al menos una persona. El grupo se confirma con al menos 5.</t>
+        </is>
+      </c>
+      <c r="G868" s="13" t="inlineStr"/>
+      <c r="H868" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I868" s="13" t="inlineStr"/>
+      <c r="J868" s="12" t="inlineStr"/>
+      <c r="K868" s="14" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L868" s="14" t="inlineStr">
+        <is>
+          <t>Código del sitio (sitio/app/grupos.js)</t>
+        </is>
+      </c>
+    </row>
+    <row r="869">
+      <c r="A869" s="15" t="inlineStr">
+        <is>
+          <t>T868</t>
+        </is>
+      </c>
+      <c r="B869" s="15" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C869" s="15" t="inlineStr">
+        <is>
+          <t>Paso 4 · confirmar</t>
+        </is>
+      </c>
+      <c r="D869" s="15" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="E869" s="15" t="inlineStr">
+        <is>
+          <t>Antes de crearlo</t>
+        </is>
+      </c>
+      <c r="F869" s="15" t="inlineStr">
+        <is>
+          <t>Se crea confirmado · Cada persona verá en «Mis trámites» la fecha, la hora y el lugar. / Se crea por confirmar · Para confirmarlo le falta …</t>
+        </is>
+      </c>
+      <c r="G869" s="13" t="inlineStr"/>
+      <c r="H869" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I869" s="13" t="inlineStr"/>
+      <c r="J869" s="15" t="inlineStr"/>
+      <c r="K869" s="16" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L869" s="16" t="inlineStr">
+        <is>
+          <t>Código del sitio (sitio/app/grupos.js)</t>
+        </is>
+      </c>
+    </row>
+    <row r="870">
+      <c r="A870" s="12" t="inlineStr">
+        <is>
+          <t>T869</t>
+        </is>
+      </c>
+      <c r="B870" s="12" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C870" s="12" t="inlineStr">
+        <is>
+          <t>Paso 4 · confirmar</t>
+        </is>
+      </c>
+      <c r="D870" s="12" t="inlineStr">
+        <is>
+          <t>Botón</t>
+        </is>
+      </c>
+      <c r="E870" s="12" t="inlineStr">
+        <is>
+          <t>Grupo nuevo</t>
+        </is>
+      </c>
+      <c r="F870" s="12" t="inlineStr">
+        <is>
+          <t>Crear el grupo · Crear sin confirmar (sólo si podría confirmarse)</t>
+        </is>
+      </c>
+      <c r="G870" s="13" t="inlineStr"/>
+      <c r="H870" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I870" s="13" t="inlineStr"/>
+      <c r="J870" s="12" t="inlineStr"/>
+      <c r="K870" s="14" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L870" s="14" t="inlineStr">
+        <is>
+          <t>Código del sitio (sitio/app/grupos.js)</t>
+        </is>
+      </c>
+    </row>
+    <row r="871">
+      <c r="A871" s="15" t="inlineStr">
+        <is>
+          <t>T870</t>
+        </is>
+      </c>
+      <c r="B871" s="15" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C871" s="15" t="inlineStr">
+        <is>
+          <t>Paso 4 · confirmar</t>
+        </is>
+      </c>
+      <c r="D871" s="15" t="inlineStr">
+        <is>
+          <t>Botón</t>
+        </is>
+      </c>
+      <c r="E871" s="15" t="inlineStr">
+        <is>
+          <t>Grupo que ya existe</t>
+        </is>
+      </c>
+      <c r="F871" s="15" t="inlineStr">
+        <is>
+          <t>Confirmar el grupo / Guardar los cambios / Guardar sin confirmar / Agregar al grupo (confirmado)</t>
+        </is>
+      </c>
+      <c r="G871" s="13" t="inlineStr"/>
+      <c r="H871" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I871" s="13" t="inlineStr"/>
+      <c r="J871" s="15" t="inlineStr"/>
+      <c r="K871" s="16" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L871" s="16" t="inlineStr">
+        <is>
+          <t>Código del sitio (sitio/app/grupos.js)</t>
+        </is>
+      </c>
+    </row>
+    <row r="872">
+      <c r="A872" s="12" t="inlineStr">
+        <is>
+          <t>T871</t>
+        </is>
+      </c>
+      <c r="B872" s="12" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C872" s="12" t="inlineStr">
+        <is>
+          <t>Paso 4 · instructor</t>
+        </is>
+      </c>
+      <c r="D872" s="12" t="inlineStr">
+        <is>
+          <t>Ayuda (cambia)</t>
+        </is>
+      </c>
+      <c r="E872" s="12" t="inlineStr">
+        <is>
+          <t>Instructor «Por asignar»</t>
+        </is>
+      </c>
+      <c r="F872" s="12" t="inlineStr">
+        <is>
+          <t>Por asignar: el grupo se crea, pero no se confirma sin instructor. La asignación de instructores la hará el área de capacitación (pendiente P92).</t>
+        </is>
+      </c>
+      <c r="G872" s="13" t="inlineStr"/>
+      <c r="H872" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I872" s="13" t="inlineStr"/>
+      <c r="J872" s="12" t="inlineStr"/>
+      <c r="K872" s="14" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L872" s="14" t="inlineStr">
+        <is>
+          <t>Código del sitio (sitio/app/grupos.js)</t>
+        </is>
+      </c>
+    </row>
+    <row r="873">
+      <c r="A873" s="15" t="inlineStr">
+        <is>
+          <t>T872</t>
+        </is>
+      </c>
+      <c r="B873" s="15" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C873" s="15" t="inlineStr">
+        <is>
+          <t>Grupos programados</t>
+        </is>
+      </c>
+      <c r="D873" s="15" t="inlineStr">
+        <is>
+          <t>Aviso</t>
+        </is>
+      </c>
+      <c r="E873" s="15" t="inlineStr">
+        <is>
+          <t>Al crear un grupo</t>
+        </is>
+      </c>
+      <c r="F873" s="15" t="inlineStr">
+        <is>
+          <t>Grupo creado y confirmado: NOMBRE / Grupo creado, por confirmar: NOMBRE · FOLIO · N personas · entrada a las 09:00 · INSTRUCTOR. · Ver la ficha del grupo · Qué sigue</t>
+        </is>
+      </c>
+      <c r="G873" s="13" t="inlineStr"/>
+      <c r="H873" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I873" s="13" t="inlineStr"/>
+      <c r="J873" s="15" t="inlineStr"/>
+      <c r="K873" s="16" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L873" s="16" t="inlineStr">
+        <is>
+          <t>Código del sitio (sitio/app/grupos.js)</t>
+        </is>
+      </c>
+    </row>
+    <row r="874">
+      <c r="A874" s="12" t="inlineStr">
+        <is>
+          <t>T873</t>
+        </is>
+      </c>
+      <c r="B874" s="12" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C874" s="12" t="inlineStr">
+        <is>
+          <t>Grupos programados</t>
+        </is>
+      </c>
+      <c r="D874" s="12" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="E874" s="12" t="inlineStr">
+        <is>
+          <t>Situación de cada grupo</t>
+        </is>
+      </c>
+      <c r="F874" s="12" t="inlineStr">
+        <is>
+          <t>En curso · día N de 5 / Confirmado / Por confirmar / Sin semana / Propuesta vencida / Confirmado · no inició</t>
+        </is>
+      </c>
+      <c r="G874" s="13" t="inlineStr"/>
+      <c r="H874" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I874" s="13" t="inlineStr"/>
+      <c r="J874" s="12" t="inlineStr"/>
+      <c r="K874" s="14" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L874" s="14" t="inlineStr">
+        <is>
+          <t>Código del sitio (sitio/app/grupos.js)</t>
+        </is>
+      </c>
+    </row>
+    <row r="875">
+      <c r="A875" s="15" t="inlineStr">
+        <is>
+          <t>T874</t>
+        </is>
+      </c>
+      <c r="B875" s="15" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C875" s="15" t="inlineStr">
+        <is>
+          <t>Grupos programados</t>
+        </is>
+      </c>
+      <c r="D875" s="15" t="inlineStr">
+        <is>
+          <t>Botón o enlace</t>
+        </is>
+      </c>
+      <c r="E875" s="15" t="inlineStr">
+        <is>
+          <t>Acciones de cada grupo</t>
+        </is>
+      </c>
+      <c r="F875" s="15" t="inlineStr">
+        <is>
+          <t>Completar con las N que más esperan · Confirmar el grupo · Elegir semana / Cambiar la semana / Elegir otra semana · Agregar personas</t>
+        </is>
+      </c>
+      <c r="G875" s="13" t="inlineStr"/>
+      <c r="H875" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I875" s="13" t="inlineStr"/>
+      <c r="J875" s="15" t="inlineStr"/>
+      <c r="K875" s="16" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L875" s="16" t="inlineStr">
+        <is>
+          <t>Código del sitio (sitio/app/grupos.js)</t>
+        </is>
+      </c>
+    </row>
+    <row r="876">
+      <c r="A876" s="12" t="inlineStr">
+        <is>
+          <t>T875</t>
+        </is>
+      </c>
+      <c r="B876" s="12" t="inlineStr">
+        <is>
+          <t>Grupos (personal)</t>
+        </is>
+      </c>
+      <c r="C876" s="12" t="inlineStr">
+        <is>
+          <t>Grupos programados</t>
+        </is>
+      </c>
+      <c r="D876" s="12" t="inlineStr">
+        <is>
+          <t>Texto</t>
+        </is>
+      </c>
+      <c r="E876" s="12" t="inlineStr">
+        <is>
+          <t>Lo que falta</t>
+        </is>
+      </c>
+      <c r="F876" s="12" t="inlineStr">
+        <is>
+          <t>Semana, N personas, hora e instructor / Confirmarlo / —</t>
+        </is>
+      </c>
+      <c r="G876" s="13" t="inlineStr"/>
+      <c r="H876" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I876" s="13" t="inlineStr"/>
+      <c r="J876" s="12" t="inlineStr"/>
+      <c r="K876" s="14" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L876" s="14" t="inlineStr">
+        <is>
+          <t>Código del sitio (sitio/app/grupos.js)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L803"/>
-  <conditionalFormatting sqref="H2:H803">
+  <autoFilter ref="A1:L876"/>
+  <conditionalFormatting sqref="H2:H876">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"OK"</formula>
     </cfRule>
@@ -41338,13 +44992,13 @@
       <formula>"Duda"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G803">
+  <conditionalFormatting sqref="G2:G876">
     <cfRule type="expression" priority="5" dxfId="4">
       <formula>AND(LEN(G2)&gt;0,H2="Pendiente")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H803" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Estado" error="Elige: Pendiente, OK, Cambiar, Quitar o Duda." type="list">
+    <dataValidation sqref="H2:H876" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Estado" error="Elige: Pendiente, OK, Cambiar, Quitar o Duda." type="list">
       <formula1>"Pendiente,OK,Cambiar,Quitar,Duda"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Hora del curso fija: sin menú «Hora de entrada» en «Grupos» ni en la ficha del grupo
Decisión de Liber del 24/10/2026: el curso es de 9:00 a 15:00 (parámetros
curso_hora_entrada y curso_hora_salida). Se quita el <select> del paso 4 de
«Grupos» y del formulario de confirmar de la ficha; el horario se muestra como
dato («Horario: de 9:00 a 15:00, de lunes a viernes») y al crear, proponer o
confirmar el grupo toma hora_entrada del parámetro, también los ficticios que
no la tenían. «Hora» sale de lo que le falta a un grupo y de los mensajes.
Esquemas grupo-crear y grupo-confirmar regenerados (sin hora_entrada; si llega,
se rechaza como campo no declarado), pruebas ajustadas, ETAPA-2-PANTALLAS e
inventario de textos al día.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YEpbunHXM4tST7Mz5ceBJ7
</commit_message>
<xml_diff>
--- a/docs/textos/inventario-textos.xlsx
+++ b/docs/textos/inventario-textos.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Textos" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Textos'!$A$1:$L$886</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Textos'!$A$1:$L$883</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -600,7 +600,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Inventario generado de la versión de prueba 0.67 · 885 textos</t>
+          <t>Inventario generado de la versión de prueba 0.68 · 882 textos</t>
         </is>
       </c>
     </row>
@@ -761,23 +761,23 @@
         </is>
       </c>
       <c r="B21" s="8">
-        <f>COUNTIF(Textos!$B$2:$B$886,A21)</f>
+        <f>COUNTIF(Textos!$B$2:$B$883,A21)</f>
         <v/>
       </c>
       <c r="C21" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$886,A21,Textos!$H$2:$H$886,"Pendiente")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$883,A21,Textos!$H$2:$H$883,"Pendiente")</f>
         <v/>
       </c>
       <c r="D21" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$886,A21,Textos!$H$2:$H$886,"OK")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$883,A21,Textos!$H$2:$H$883,"OK")</f>
         <v/>
       </c>
       <c r="E21" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$886,A21,Textos!$H$2:$H$886,"Cambiar")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$883,A21,Textos!$H$2:$H$883,"Cambiar")</f>
         <v/>
       </c>
       <c r="F21" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$886,A21,Textos!$H$2:$H$886,"Quitar")+COUNTIFS(Textos!$B$2:$B$886,A21,Textos!$H$2:$H$886,"Duda")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$883,A21,Textos!$H$2:$H$883,"Quitar")+COUNTIFS(Textos!$B$2:$B$883,A21,Textos!$H$2:$H$883,"Duda")</f>
         <v/>
       </c>
     </row>
@@ -788,23 +788,23 @@
         </is>
       </c>
       <c r="B22" s="8">
-        <f>COUNTIF(Textos!$B$2:$B$886,A22)</f>
+        <f>COUNTIF(Textos!$B$2:$B$883,A22)</f>
         <v/>
       </c>
       <c r="C22" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$886,A22,Textos!$H$2:$H$886,"Pendiente")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$883,A22,Textos!$H$2:$H$883,"Pendiente")</f>
         <v/>
       </c>
       <c r="D22" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$886,A22,Textos!$H$2:$H$886,"OK")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$883,A22,Textos!$H$2:$H$883,"OK")</f>
         <v/>
       </c>
       <c r="E22" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$886,A22,Textos!$H$2:$H$886,"Cambiar")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$883,A22,Textos!$H$2:$H$883,"Cambiar")</f>
         <v/>
       </c>
       <c r="F22" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$886,A22,Textos!$H$2:$H$886,"Quitar")+COUNTIFS(Textos!$B$2:$B$886,A22,Textos!$H$2:$H$886,"Duda")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$883,A22,Textos!$H$2:$H$883,"Quitar")+COUNTIFS(Textos!$B$2:$B$883,A22,Textos!$H$2:$H$883,"Duda")</f>
         <v/>
       </c>
     </row>
@@ -815,23 +815,23 @@
         </is>
       </c>
       <c r="B23" s="8">
-        <f>COUNTIF(Textos!$B$2:$B$886,A23)</f>
+        <f>COUNTIF(Textos!$B$2:$B$883,A23)</f>
         <v/>
       </c>
       <c r="C23" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$886,A23,Textos!$H$2:$H$886,"Pendiente")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$883,A23,Textos!$H$2:$H$883,"Pendiente")</f>
         <v/>
       </c>
       <c r="D23" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$886,A23,Textos!$H$2:$H$886,"OK")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$883,A23,Textos!$H$2:$H$883,"OK")</f>
         <v/>
       </c>
       <c r="E23" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$886,A23,Textos!$H$2:$H$886,"Cambiar")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$883,A23,Textos!$H$2:$H$883,"Cambiar")</f>
         <v/>
       </c>
       <c r="F23" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$886,A23,Textos!$H$2:$H$886,"Quitar")+COUNTIFS(Textos!$B$2:$B$886,A23,Textos!$H$2:$H$886,"Duda")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$883,A23,Textos!$H$2:$H$883,"Quitar")+COUNTIFS(Textos!$B$2:$B$883,A23,Textos!$H$2:$H$883,"Duda")</f>
         <v/>
       </c>
     </row>
@@ -842,23 +842,23 @@
         </is>
       </c>
       <c r="B24" s="8">
-        <f>COUNTIF(Textos!$B$2:$B$886,A24)</f>
+        <f>COUNTIF(Textos!$B$2:$B$883,A24)</f>
         <v/>
       </c>
       <c r="C24" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$886,A24,Textos!$H$2:$H$886,"Pendiente")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$883,A24,Textos!$H$2:$H$883,"Pendiente")</f>
         <v/>
       </c>
       <c r="D24" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$886,A24,Textos!$H$2:$H$886,"OK")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$883,A24,Textos!$H$2:$H$883,"OK")</f>
         <v/>
       </c>
       <c r="E24" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$886,A24,Textos!$H$2:$H$886,"Cambiar")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$883,A24,Textos!$H$2:$H$883,"Cambiar")</f>
         <v/>
       </c>
       <c r="F24" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$886,A24,Textos!$H$2:$H$886,"Quitar")+COUNTIFS(Textos!$B$2:$B$886,A24,Textos!$H$2:$H$886,"Duda")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$883,A24,Textos!$H$2:$H$883,"Quitar")+COUNTIFS(Textos!$B$2:$B$883,A24,Textos!$H$2:$H$883,"Duda")</f>
         <v/>
       </c>
     </row>
@@ -869,23 +869,23 @@
         </is>
       </c>
       <c r="B25" s="8">
-        <f>COUNTIF(Textos!$B$2:$B$886,A25)</f>
+        <f>COUNTIF(Textos!$B$2:$B$883,A25)</f>
         <v/>
       </c>
       <c r="C25" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$886,A25,Textos!$H$2:$H$886,"Pendiente")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$883,A25,Textos!$H$2:$H$883,"Pendiente")</f>
         <v/>
       </c>
       <c r="D25" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$886,A25,Textos!$H$2:$H$886,"OK")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$883,A25,Textos!$H$2:$H$883,"OK")</f>
         <v/>
       </c>
       <c r="E25" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$886,A25,Textos!$H$2:$H$886,"Cambiar")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$883,A25,Textos!$H$2:$H$883,"Cambiar")</f>
         <v/>
       </c>
       <c r="F25" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$886,A25,Textos!$H$2:$H$886,"Quitar")+COUNTIFS(Textos!$B$2:$B$886,A25,Textos!$H$2:$H$886,"Duda")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$883,A25,Textos!$H$2:$H$883,"Quitar")+COUNTIFS(Textos!$B$2:$B$883,A25,Textos!$H$2:$H$883,"Duda")</f>
         <v/>
       </c>
     </row>
@@ -896,23 +896,23 @@
         </is>
       </c>
       <c r="B26" s="8">
-        <f>COUNTIF(Textos!$B$2:$B$886,A26)</f>
+        <f>COUNTIF(Textos!$B$2:$B$883,A26)</f>
         <v/>
       </c>
       <c r="C26" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$886,A26,Textos!$H$2:$H$886,"Pendiente")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$883,A26,Textos!$H$2:$H$883,"Pendiente")</f>
         <v/>
       </c>
       <c r="D26" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$886,A26,Textos!$H$2:$H$886,"OK")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$883,A26,Textos!$H$2:$H$883,"OK")</f>
         <v/>
       </c>
       <c r="E26" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$886,A26,Textos!$H$2:$H$886,"Cambiar")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$883,A26,Textos!$H$2:$H$883,"Cambiar")</f>
         <v/>
       </c>
       <c r="F26" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$886,A26,Textos!$H$2:$H$886,"Quitar")+COUNTIFS(Textos!$B$2:$B$886,A26,Textos!$H$2:$H$886,"Duda")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$883,A26,Textos!$H$2:$H$883,"Quitar")+COUNTIFS(Textos!$B$2:$B$883,A26,Textos!$H$2:$H$883,"Duda")</f>
         <v/>
       </c>
     </row>
@@ -923,23 +923,23 @@
         </is>
       </c>
       <c r="B27" s="8">
-        <f>COUNTIF(Textos!$B$2:$B$886,A27)</f>
+        <f>COUNTIF(Textos!$B$2:$B$883,A27)</f>
         <v/>
       </c>
       <c r="C27" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$886,A27,Textos!$H$2:$H$886,"Pendiente")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$883,A27,Textos!$H$2:$H$883,"Pendiente")</f>
         <v/>
       </c>
       <c r="D27" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$886,A27,Textos!$H$2:$H$886,"OK")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$883,A27,Textos!$H$2:$H$883,"OK")</f>
         <v/>
       </c>
       <c r="E27" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$886,A27,Textos!$H$2:$H$886,"Cambiar")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$883,A27,Textos!$H$2:$H$883,"Cambiar")</f>
         <v/>
       </c>
       <c r="F27" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$886,A27,Textos!$H$2:$H$886,"Quitar")+COUNTIFS(Textos!$B$2:$B$886,A27,Textos!$H$2:$H$886,"Duda")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$883,A27,Textos!$H$2:$H$883,"Quitar")+COUNTIFS(Textos!$B$2:$B$883,A27,Textos!$H$2:$H$883,"Duda")</f>
         <v/>
       </c>
     </row>
@@ -950,23 +950,23 @@
         </is>
       </c>
       <c r="B28" s="8">
-        <f>COUNTIF(Textos!$B$2:$B$886,A28)</f>
+        <f>COUNTIF(Textos!$B$2:$B$883,A28)</f>
         <v/>
       </c>
       <c r="C28" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$886,A28,Textos!$H$2:$H$886,"Pendiente")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$883,A28,Textos!$H$2:$H$883,"Pendiente")</f>
         <v/>
       </c>
       <c r="D28" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$886,A28,Textos!$H$2:$H$886,"OK")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$883,A28,Textos!$H$2:$H$883,"OK")</f>
         <v/>
       </c>
       <c r="E28" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$886,A28,Textos!$H$2:$H$886,"Cambiar")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$883,A28,Textos!$H$2:$H$883,"Cambiar")</f>
         <v/>
       </c>
       <c r="F28" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$886,A28,Textos!$H$2:$H$886,"Quitar")+COUNTIFS(Textos!$B$2:$B$886,A28,Textos!$H$2:$H$886,"Duda")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$883,A28,Textos!$H$2:$H$883,"Quitar")+COUNTIFS(Textos!$B$2:$B$883,A28,Textos!$H$2:$H$883,"Duda")</f>
         <v/>
       </c>
     </row>
@@ -977,23 +977,23 @@
         </is>
       </c>
       <c r="B29" s="8">
-        <f>COUNTIF(Textos!$B$2:$B$886,A29)</f>
+        <f>COUNTIF(Textos!$B$2:$B$883,A29)</f>
         <v/>
       </c>
       <c r="C29" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$886,A29,Textos!$H$2:$H$886,"Pendiente")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$883,A29,Textos!$H$2:$H$883,"Pendiente")</f>
         <v/>
       </c>
       <c r="D29" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$886,A29,Textos!$H$2:$H$886,"OK")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$883,A29,Textos!$H$2:$H$883,"OK")</f>
         <v/>
       </c>
       <c r="E29" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$886,A29,Textos!$H$2:$H$886,"Cambiar")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$883,A29,Textos!$H$2:$H$883,"Cambiar")</f>
         <v/>
       </c>
       <c r="F29" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$886,A29,Textos!$H$2:$H$886,"Quitar")+COUNTIFS(Textos!$B$2:$B$886,A29,Textos!$H$2:$H$886,"Duda")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$883,A29,Textos!$H$2:$H$883,"Quitar")+COUNTIFS(Textos!$B$2:$B$883,A29,Textos!$H$2:$H$883,"Duda")</f>
         <v/>
       </c>
     </row>
@@ -1004,23 +1004,23 @@
         </is>
       </c>
       <c r="B30" s="8">
-        <f>COUNTIF(Textos!$B$2:$B$886,A30)</f>
+        <f>COUNTIF(Textos!$B$2:$B$883,A30)</f>
         <v/>
       </c>
       <c r="C30" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$886,A30,Textos!$H$2:$H$886,"Pendiente")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$883,A30,Textos!$H$2:$H$883,"Pendiente")</f>
         <v/>
       </c>
       <c r="D30" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$886,A30,Textos!$H$2:$H$886,"OK")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$883,A30,Textos!$H$2:$H$883,"OK")</f>
         <v/>
       </c>
       <c r="E30" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$886,A30,Textos!$H$2:$H$886,"Cambiar")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$883,A30,Textos!$H$2:$H$883,"Cambiar")</f>
         <v/>
       </c>
       <c r="F30" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$886,A30,Textos!$H$2:$H$886,"Quitar")+COUNTIFS(Textos!$B$2:$B$886,A30,Textos!$H$2:$H$886,"Duda")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$883,A30,Textos!$H$2:$H$883,"Quitar")+COUNTIFS(Textos!$B$2:$B$883,A30,Textos!$H$2:$H$883,"Duda")</f>
         <v/>
       </c>
     </row>
@@ -1031,23 +1031,23 @@
         </is>
       </c>
       <c r="B31" s="8">
-        <f>COUNTIF(Textos!$B$2:$B$886,A31)</f>
+        <f>COUNTIF(Textos!$B$2:$B$883,A31)</f>
         <v/>
       </c>
       <c r="C31" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$886,A31,Textos!$H$2:$H$886,"Pendiente")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$883,A31,Textos!$H$2:$H$883,"Pendiente")</f>
         <v/>
       </c>
       <c r="D31" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$886,A31,Textos!$H$2:$H$886,"OK")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$883,A31,Textos!$H$2:$H$883,"OK")</f>
         <v/>
       </c>
       <c r="E31" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$886,A31,Textos!$H$2:$H$886,"Cambiar")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$883,A31,Textos!$H$2:$H$883,"Cambiar")</f>
         <v/>
       </c>
       <c r="F31" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$886,A31,Textos!$H$2:$H$886,"Quitar")+COUNTIFS(Textos!$B$2:$B$886,A31,Textos!$H$2:$H$886,"Duda")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$883,A31,Textos!$H$2:$H$883,"Quitar")+COUNTIFS(Textos!$B$2:$B$883,A31,Textos!$H$2:$H$883,"Duda")</f>
         <v/>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L886"/>
+  <dimension ref="A1:L883"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -43744,7 +43744,7 @@
       </c>
       <c r="D852" s="12" t="inlineStr">
         <is>
-          <t>Pregunta</t>
+          <t>Botón o enlace</t>
         </is>
       </c>
       <c r="E852" s="12" t="inlineStr">
@@ -43754,7 +43754,7 @@
       </c>
       <c r="F852" s="12" t="inlineStr">
         <is>
-          <t>Hora de entrada</t>
+          <t>Atrás</t>
         </is>
       </c>
       <c r="G852" s="13" t="inlineStr"/>
@@ -43794,7 +43794,7 @@
       </c>
       <c r="D853" s="15" t="inlineStr">
         <is>
-          <t>Ayuda</t>
+          <t>Botón o enlace</t>
         </is>
       </c>
       <c r="E853" s="15" t="inlineStr">
@@ -43804,7 +43804,7 @@
       </c>
       <c r="F853" s="15" t="inlineStr">
         <is>
-          <t>El curso es de 9:00 a 15:00 todos sus días.</t>
+          <t>Crear sin confirmar</t>
         </is>
       </c>
       <c r="G853" s="13" t="inlineStr"/>
@@ -43844,7 +43844,7 @@
       </c>
       <c r="D854" s="12" t="inlineStr">
         <is>
-          <t>Indicación de lista</t>
+          <t>Botón o enlace</t>
         </is>
       </c>
       <c r="E854" s="12" t="inlineStr">
@@ -43854,7 +43854,7 @@
       </c>
       <c r="F854" s="12" t="inlineStr">
         <is>
-          <t>Elija</t>
+          <t>Crear el grupo</t>
         </is>
       </c>
       <c r="G854" s="13" t="inlineStr"/>
@@ -43889,12 +43889,12 @@
       </c>
       <c r="C855" s="15" t="inlineStr">
         <is>
-          <t>Confirmar</t>
+          <t>Grupos programados</t>
         </is>
       </c>
       <c r="D855" s="15" t="inlineStr">
         <is>
-          <t>Botón o enlace</t>
+          <t>Subtítulo</t>
         </is>
       </c>
       <c r="E855" s="15" t="inlineStr">
@@ -43904,7 +43904,7 @@
       </c>
       <c r="F855" s="15" t="inlineStr">
         <is>
-          <t>Atrás</t>
+          <t>Grupos programados</t>
         </is>
       </c>
       <c r="G855" s="13" t="inlineStr"/>
@@ -43939,12 +43939,12 @@
       </c>
       <c r="C856" s="12" t="inlineStr">
         <is>
-          <t>Confirmar</t>
+          <t>Grupos programados</t>
         </is>
       </c>
       <c r="D856" s="12" t="inlineStr">
         <is>
-          <t>Botón o enlace</t>
+          <t>Introducción</t>
         </is>
       </c>
       <c r="E856" s="12" t="inlineStr">
@@ -43954,7 +43954,7 @@
       </c>
       <c r="F856" s="12" t="inlineStr">
         <is>
-          <t>Crear sin confirmar</t>
+          <t>Por curso: los grupos por confirmar, confirmados y en curso, con lo que les falta.</t>
         </is>
       </c>
       <c r="G856" s="13" t="inlineStr"/>
@@ -43989,12 +43989,12 @@
       </c>
       <c r="C857" s="15" t="inlineStr">
         <is>
-          <t>Confirmar</t>
+          <t>Grupos programados</t>
         </is>
       </c>
       <c r="D857" s="15" t="inlineStr">
         <is>
-          <t>Botón o enlace</t>
+          <t>Título desplegable</t>
         </is>
       </c>
       <c r="E857" s="15" t="inlineStr">
@@ -44004,7 +44004,7 @@
       </c>
       <c r="F857" s="15" t="inlineStr">
         <is>
-          <t>Crear el grupo</t>
+          <t>Grupos que ya terminaron</t>
         </is>
       </c>
       <c r="G857" s="13" t="inlineStr"/>
@@ -44044,7 +44044,7 @@
       </c>
       <c r="D858" s="12" t="inlineStr">
         <is>
-          <t>Subtítulo</t>
+          <t>Ayuda</t>
         </is>
       </c>
       <c r="E858" s="12" t="inlineStr">
@@ -44054,7 +44054,7 @@
       </c>
       <c r="F858" s="12" t="inlineStr">
         <is>
-          <t>Grupos programados</t>
+          <t>Los cuatro cursos nunca se mezclan; un grupo se confirma con al menos 5 personas e instructor, y recibe hasta 25. Pendiente (P92): quién arma los grupos (hoy, el perfil de revisión y cotejo) y quién asigna a los instructores.</t>
         </is>
       </c>
       <c r="G858" s="13" t="inlineStr"/>
@@ -44084,27 +44084,27 @@
       </c>
       <c r="B859" s="15" t="inlineStr">
         <is>
-          <t>Grupos (personal)</t>
+          <t>Reposición de tu credencial</t>
         </is>
       </c>
       <c r="C859" s="15" t="inlineStr">
         <is>
-          <t>Grupos programados</t>
+          <t>Resultado</t>
         </is>
       </c>
       <c r="D859" s="15" t="inlineStr">
         <is>
-          <t>Introducción</t>
+          <t>Título</t>
         </is>
       </c>
       <c r="E859" s="15" t="inlineStr">
         <is>
-          <t>Siempre</t>
+          <t>Al pedirla o al cargar el acta corregida</t>
         </is>
       </c>
       <c r="F859" s="15" t="inlineStr">
         <is>
-          <t>Por curso: los grupos por confirmar, confirmados y en curso, con lo que les falta.</t>
+          <t>Recibimos tu solicitud de reposición · Recibimos tu acta corregida</t>
         </is>
       </c>
       <c r="G859" s="13" t="inlineStr"/>
@@ -44117,12 +44117,12 @@
       <c r="J859" s="15" t="inlineStr"/>
       <c r="K859" s="16" t="inlineStr">
         <is>
-          <t>Personal de la Secretaría</t>
+          <t>Persona solicitante</t>
         </is>
       </c>
       <c r="L859" s="16" t="inlineStr">
         <is>
-          <t>Página (sitio/grupos.html)</t>
+          <t>Código del sitio (sitio/app/reposicion.js)</t>
         </is>
       </c>
     </row>
@@ -44134,27 +44134,27 @@
       </c>
       <c r="B860" s="12" t="inlineStr">
         <is>
-          <t>Grupos (personal)</t>
+          <t>Reposición de tu credencial</t>
         </is>
       </c>
       <c r="C860" s="12" t="inlineStr">
         <is>
-          <t>Grupos programados</t>
+          <t>Resultado</t>
         </is>
       </c>
       <c r="D860" s="12" t="inlineStr">
         <is>
-          <t>Título desplegable</t>
+          <t>Pasos</t>
         </is>
       </c>
       <c r="E860" s="12" t="inlineStr">
         <is>
-          <t>Siempre</t>
+          <t>Al pedirla</t>
         </is>
       </c>
       <c r="F860" s="12" t="inlineStr">
         <is>
-          <t>Grupos que ya terminaron</t>
+          <t>La Secretaría revisa tu acta. · Te indica en «Mis trámites» si debes corregir algo o, si está completa, cuánto pagar. · Pagas la cuota de reposición y recoges tu credencial en la oficina del Vivero Nezahualcóyotl, con el mismo número y la misma vigencia.</t>
         </is>
       </c>
       <c r="G860" s="13" t="inlineStr"/>
@@ -44167,12 +44167,12 @@
       <c r="J860" s="12" t="inlineStr"/>
       <c r="K860" s="14" t="inlineStr">
         <is>
-          <t>Personal de la Secretaría</t>
+          <t>Persona solicitante</t>
         </is>
       </c>
       <c r="L860" s="14" t="inlineStr">
         <is>
-          <t>Página (sitio/grupos.html)</t>
+          <t>Código del sitio (sitio/app/reposicion.js)</t>
         </is>
       </c>
     </row>
@@ -44184,27 +44184,27 @@
       </c>
       <c r="B861" s="15" t="inlineStr">
         <is>
-          <t>Grupos (personal)</t>
+          <t>Reposición de tu credencial</t>
         </is>
       </c>
       <c r="C861" s="15" t="inlineStr">
         <is>
-          <t>Grupos programados</t>
+          <t>Acreditación</t>
         </is>
       </c>
       <c r="D861" s="15" t="inlineStr">
         <is>
-          <t>Ayuda</t>
+          <t>Error</t>
         </is>
       </c>
       <c r="E861" s="15" t="inlineStr">
         <is>
-          <t>Siempre</t>
+          <t>Credencial del sistema que todavía no se entrega</t>
         </is>
       </c>
       <c r="F861" s="15" t="inlineStr">
         <is>
-          <t>Los cuatro cursos nunca se mezclan; un grupo se confirma con al menos 5 personas, hora de entrada e instructor, y recibe hasta 25. Pendiente (P92): quién arma los grupos (hoy, el perfil de revisión y cotejo) y quién asigna a los instructores.</t>
+          <t>Tu credencial todavía no se te entrega: recógela en la oficina del Vivero. La reposición es para una credencial que ya recibiste y perdiste o te robaron.</t>
         </is>
       </c>
       <c r="G861" s="13" t="inlineStr"/>
@@ -44217,12 +44217,12 @@
       <c r="J861" s="15" t="inlineStr"/>
       <c r="K861" s="16" t="inlineStr">
         <is>
-          <t>Personal de la Secretaría</t>
+          <t>Persona solicitante</t>
         </is>
       </c>
       <c r="L861" s="16" t="inlineStr">
         <is>
-          <t>Página (sitio/grupos.html)</t>
+          <t>Código del sitio (sitio/app/reposicion.js)</t>
         </is>
       </c>
     </row>
@@ -44234,27 +44234,27 @@
       </c>
       <c r="B862" s="12" t="inlineStr">
         <is>
-          <t>Reposición de tu credencial</t>
+          <t>Grupos (personal)</t>
         </is>
       </c>
       <c r="C862" s="12" t="inlineStr">
         <is>
-          <t>Resultado</t>
+          <t>Cabecera</t>
         </is>
       </c>
       <c r="D862" s="12" t="inlineStr">
         <is>
-          <t>Título</t>
+          <t>Texto</t>
         </is>
       </c>
       <c r="E862" s="12" t="inlineStr">
         <is>
-          <t>Al pedirla o al cargar el acta corregida</t>
+          <t>Siempre</t>
         </is>
       </c>
       <c r="F862" s="12" t="inlineStr">
         <is>
-          <t>Recibimos tu solicitud de reposición · Recibimos tu acta corregida</t>
+          <t>Hoy es DÍA N de MES de AAAA. Arme un grupo en cuatro pasos: el curso, la semana, quiénes van y confirmar.</t>
         </is>
       </c>
       <c r="G862" s="13" t="inlineStr"/>
@@ -44267,12 +44267,12 @@
       <c r="J862" s="12" t="inlineStr"/>
       <c r="K862" s="14" t="inlineStr">
         <is>
-          <t>Persona solicitante</t>
+          <t>Personal de la Secretaría</t>
         </is>
       </c>
       <c r="L862" s="14" t="inlineStr">
         <is>
-          <t>Código del sitio (sitio/app/reposicion.js)</t>
+          <t>Código del sitio (sitio/app/grupos.js)</t>
         </is>
       </c>
     </row>
@@ -44284,27 +44284,27 @@
       </c>
       <c r="B863" s="15" t="inlineStr">
         <is>
-          <t>Reposición de tu credencial</t>
+          <t>Grupos (personal)</t>
         </is>
       </c>
       <c r="C863" s="15" t="inlineStr">
         <is>
-          <t>Resultado</t>
+          <t>Paso 1 · el curso</t>
         </is>
       </c>
       <c r="D863" s="15" t="inlineStr">
         <is>
-          <t>Pasos</t>
+          <t>Texto</t>
         </is>
       </c>
       <c r="E863" s="15" t="inlineStr">
         <is>
-          <t>Al pedirla</t>
+          <t>En cada curso</t>
         </is>
       </c>
       <c r="F863" s="15" t="inlineStr">
         <is>
-          <t>La Secretaría revisa tu acta. · Te indica en «Mis trámites» si debes corregir algo o, si está completa, cuánto pagar. · Pagas la cuota de reposición y recoges tu credencial en la oficina del Vivero Nezahualcóyotl, con el mismo número y la misma vigencia.</t>
+          <t>N personas en espera · N esperan 15 días o más · N ya vencidas · Falta gente para un grupo (mínimo 5) / Alcanza para N grupos nuevos de hasta 25 / Nadie espera por ahora</t>
         </is>
       </c>
       <c r="G863" s="13" t="inlineStr"/>
@@ -44317,12 +44317,12 @@
       <c r="J863" s="15" t="inlineStr"/>
       <c r="K863" s="16" t="inlineStr">
         <is>
-          <t>Persona solicitante</t>
+          <t>Personal de la Secretaría</t>
         </is>
       </c>
       <c r="L863" s="16" t="inlineStr">
         <is>
-          <t>Código del sitio (sitio/app/reposicion.js)</t>
+          <t>Código del sitio (sitio/app/grupos.js)</t>
         </is>
       </c>
     </row>
@@ -44334,27 +44334,27 @@
       </c>
       <c r="B864" s="12" t="inlineStr">
         <is>
-          <t>Reposición de tu credencial</t>
+          <t>Grupos (personal)</t>
         </is>
       </c>
       <c r="C864" s="12" t="inlineStr">
         <is>
-          <t>Acreditación</t>
+          <t>Paso 2 · la semana</t>
         </is>
       </c>
       <c r="D864" s="12" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Texto</t>
         </is>
       </c>
       <c r="E864" s="12" t="inlineStr">
         <is>
-          <t>Credencial del sistema que todavía no se entrega</t>
+          <t>Siempre</t>
         </is>
       </c>
       <c r="F864" s="12" t="inlineStr">
         <is>
-          <t>Tu credencial todavía no se te entrega: recógela en la oficina del Vivero. La reposición es para una credencial que ya recibiste y perdiste o te robaron.</t>
+          <t>CURSO · lunes a viernes, de 9:00 a 15:00 (o «un día, de 9:00 a 15:00»). Puede haber 2 grupos al mismo tiempo, de cualquier curso; el curso empieza al menos 7 días después de confirmarlo.</t>
         </is>
       </c>
       <c r="G864" s="13" t="inlineStr"/>
@@ -44367,12 +44367,12 @@
       <c r="J864" s="12" t="inlineStr"/>
       <c r="K864" s="14" t="inlineStr">
         <is>
-          <t>Persona solicitante</t>
+          <t>Personal de la Secretaría</t>
         </is>
       </c>
       <c r="L864" s="14" t="inlineStr">
         <is>
-          <t>Código del sitio (sitio/app/reposicion.js)</t>
+          <t>Código del sitio (sitio/app/grupos.js)</t>
         </is>
       </c>
     </row>
@@ -44389,22 +44389,22 @@
       </c>
       <c r="C865" s="15" t="inlineStr">
         <is>
-          <t>Cabecera</t>
+          <t>Paso 2 · columna «Semana»</t>
         </is>
       </c>
       <c r="D865" s="15" t="inlineStr">
         <is>
-          <t>Texto</t>
+          <t>Botón</t>
         </is>
       </c>
       <c r="E865" s="15" t="inlineStr">
         <is>
-          <t>Siempre</t>
+          <t>Semana que se puede elegir</t>
         </is>
       </c>
       <c r="F865" s="15" t="inlineStr">
         <is>
-          <t>Hoy es DÍA N de MES de AAAA. Arme un grupo en cuatro pasos: el curso, la semana, quiénes van y confirmar.</t>
+          <t>Libre · 2 lugares libres / 1 lugar libre de 2 (elegida: «Elegida»). Nombre para el lector: «Elegir la semana del 2 al 6 de noviembre de 2026: 2 lugares libres»</t>
         </is>
       </c>
       <c r="G865" s="13" t="inlineStr"/>
@@ -44439,22 +44439,22 @@
       </c>
       <c r="C866" s="12" t="inlineStr">
         <is>
-          <t>Paso 1 · el curso</t>
+          <t>Paso 2 · columna «Semana»</t>
         </is>
       </c>
       <c r="D866" s="12" t="inlineStr">
         <is>
-          <t>Texto</t>
+          <t>Estado</t>
         </is>
       </c>
       <c r="E866" s="12" t="inlineStr">
         <is>
-          <t>En cada curso</t>
+          <t>Semana que no se puede elegir</t>
         </is>
       </c>
       <c r="F866" s="12" t="inlineStr">
         <is>
-          <t>N personas en espera · N esperan 15 días o más · N ya vencidas · Falta gente para un grupo (mínimo 5) / Alcanza para N grupos nuevos de hasta 25 / Nadie espera por ahora</t>
+          <t>No disponible · Ya pasó / Ya empezó / Faltan menos de 7 días / Ya hay 2 grupos / Día inhábil / Falta más de un año</t>
         </is>
       </c>
       <c r="G866" s="13" t="inlineStr"/>
@@ -44489,22 +44489,22 @@
       </c>
       <c r="C867" s="15" t="inlineStr">
         <is>
-          <t>Paso 2 · la semana</t>
+          <t>Paso 2 · calendario</t>
         </is>
       </c>
       <c r="D867" s="15" t="inlineStr">
         <is>
-          <t>Texto</t>
+          <t>Etiqueta</t>
         </is>
       </c>
       <c r="E867" s="15" t="inlineStr">
         <is>
-          <t>Siempre</t>
+          <t>En los días</t>
         </is>
       </c>
       <c r="F867" s="15" t="inlineStr">
         <is>
-          <t>CURSO · lunes a viernes, de 9:00 a 15:00 (o «un día, de 9:00 a 15:00»). Puede haber 2 grupos al mismo tiempo, de cualquier curso; el curso empieza al menos 7 días después de confirmarlo.</t>
+          <t>G-AAAA-NNN (folio, el primer día) · Examen (el último) · Nuevo grupo (la semana elegida) · Hoy · Inhábil</t>
         </is>
       </c>
       <c r="G867" s="13" t="inlineStr"/>
@@ -44539,22 +44539,22 @@
       </c>
       <c r="C868" s="12" t="inlineStr">
         <is>
-          <t>Paso 2 · columna «Semana»</t>
+          <t>Paso 2 · semana elegida</t>
         </is>
       </c>
       <c r="D868" s="12" t="inlineStr">
         <is>
-          <t>Botón</t>
+          <t>Texto</t>
         </is>
       </c>
       <c r="E868" s="12" t="inlineStr">
         <is>
-          <t>Semana que se puede elegir</t>
+          <t>Con una semana elegida</t>
         </is>
       </c>
       <c r="F868" s="12" t="inlineStr">
         <is>
-          <t>Libre · 2 lugares libres / 1 lugar libre de 2 (elegida: «Elegida»). Nombre para el lector: «Elegir la semana del 2 al 6 de noviembre de 2026: 2 lugares libres»</t>
+          <t>Del 2 al 6 de noviembre · Del lunes 2 de noviembre de 2026 al viernes 6 de noviembre de 2026, de 9:00 a 15:00. El viernes, repaso de conocimientos y examen final en el PILARES. (Curso de un día: «El DÍA…, de 9:00 a 15:00, con el examen ese mismo día en el PILARES».)</t>
         </is>
       </c>
       <c r="G868" s="13" t="inlineStr"/>
@@ -44589,22 +44589,22 @@
       </c>
       <c r="C869" s="15" t="inlineStr">
         <is>
-          <t>Paso 2 · columna «Semana»</t>
+          <t>Paso 2 · semana elegida</t>
         </is>
       </c>
       <c r="D869" s="15" t="inlineStr">
         <is>
-          <t>Estado</t>
+          <t>Texto</t>
         </is>
       </c>
       <c r="E869" s="15" t="inlineStr">
         <is>
-          <t>Semana que no se puede elegir</t>
+          <t>Sin semana</t>
         </is>
       </c>
       <c r="F869" s="15" t="inlineStr">
         <is>
-          <t>No disponible · Ya pasó / Ya empezó / Faltan menos de 7 días / Ya hay 2 grupos / Día inhábil / Falta más de un año</t>
+          <t>Ninguna todavía · Toque «Libre» en la semana que quiere. (Grupo que ya existe: «Sin semana todavía · … o siga sin semana: el grupo la conserva como está».)</t>
         </is>
       </c>
       <c r="G869" s="13" t="inlineStr"/>
@@ -44639,22 +44639,22 @@
       </c>
       <c r="C870" s="12" t="inlineStr">
         <is>
-          <t>Paso 2 · calendario</t>
+          <t>Paso 2</t>
         </is>
       </c>
       <c r="D870" s="12" t="inlineStr">
         <is>
-          <t>Etiqueta</t>
+          <t>Error</t>
         </is>
       </c>
       <c r="E870" s="12" t="inlineStr">
         <is>
-          <t>En los días</t>
+          <t>Siguiente sin semana</t>
         </is>
       </c>
       <c r="F870" s="12" t="inlineStr">
         <is>
-          <t>G-AAAA-NNN (folio, el primer día) · Examen (el último) · Nuevo grupo (la semana elegida) · Hoy · Inhábil</t>
+          <t>Elija una semana libre en el calendario: toque «Libre» en la semana que quiere.</t>
         </is>
       </c>
       <c r="G870" s="13" t="inlineStr"/>
@@ -44689,22 +44689,22 @@
       </c>
       <c r="C871" s="15" t="inlineStr">
         <is>
-          <t>Paso 2 · semana elegida</t>
+          <t>Paso 2</t>
         </is>
       </c>
       <c r="D871" s="15" t="inlineStr">
         <is>
-          <t>Texto</t>
+          <t>Aviso</t>
         </is>
       </c>
       <c r="E871" s="15" t="inlineStr">
         <is>
-          <t>Con una semana elegida</t>
+          <t>Al tocar un día que no se puede</t>
         </is>
       </c>
       <c r="F871" s="15" t="inlineStr">
         <is>
-          <t>Del 2 al 6 de noviembre · Del lunes 2 de noviembre de 2026 al viernes 6 de noviembre de 2026, de 9:00 a 15:00. El viernes, repaso de conocimientos y examen final en el PILARES. (Curso de un día: «El DÍA…, de 9:00 a 15:00, con el examen ese mismo día en el PILARES».)</t>
+          <t>El DÍA no se puede: RAZÓN.</t>
         </is>
       </c>
       <c r="G871" s="13" t="inlineStr"/>
@@ -44739,7 +44739,7 @@
       </c>
       <c r="C872" s="12" t="inlineStr">
         <is>
-          <t>Paso 2 · semana elegida</t>
+          <t>Paso 3 · quiénes van</t>
         </is>
       </c>
       <c r="D872" s="12" t="inlineStr">
@@ -44749,12 +44749,12 @@
       </c>
       <c r="E872" s="12" t="inlineStr">
         <is>
-          <t>Sin semana</t>
+          <t>Grupo nuevo</t>
         </is>
       </c>
       <c r="F872" s="12" t="inlineStr">
         <is>
-          <t>Ninguna todavía · Toque «Libre» en la semana que quiere. (Grupo que ya existe: «Sin semana todavía · … o siga sin semana: el grupo la conserva como está».)</t>
+          <t>Se proponen las N personas que más esperan, primero las prioritarias y las de una misma institución de gobierno juntas. Quite o agregue a quien haga falta.</t>
         </is>
       </c>
       <c r="G872" s="13" t="inlineStr"/>
@@ -44789,22 +44789,22 @@
       </c>
       <c r="C873" s="15" t="inlineStr">
         <is>
-          <t>Paso 2</t>
+          <t>Paso 3 · quiénes van</t>
         </is>
       </c>
       <c r="D873" s="15" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Texto</t>
         </is>
       </c>
       <c r="E873" s="15" t="inlineStr">
         <is>
-          <t>Siguiente sin semana</t>
+          <t>Siempre</t>
         </is>
       </c>
       <c r="F873" s="15" t="inlineStr">
         <is>
-          <t>Elija una semana libre en el calendario: toque «Libre» en la semana que quiere.</t>
+          <t>N de 25 lugares · se confirma con al menos 5 personas</t>
         </is>
       </c>
       <c r="G873" s="13" t="inlineStr"/>
@@ -44839,22 +44839,22 @@
       </c>
       <c r="C874" s="12" t="inlineStr">
         <is>
-          <t>Paso 2</t>
+          <t>Paso 3 · quiénes van</t>
         </is>
       </c>
       <c r="D874" s="12" t="inlineStr">
         <is>
-          <t>Aviso</t>
+          <t>Plegable</t>
         </is>
       </c>
       <c r="E874" s="12" t="inlineStr">
         <is>
-          <t>Al tocar un día que no se puede</t>
+          <t>Con más en espera que las propuestas</t>
         </is>
       </c>
       <c r="F874" s="12" t="inlineStr">
         <is>
-          <t>El DÍA no se puede: RAZÓN.</t>
+          <t>Cambiar a quiénes van (N más en espera)</t>
         </is>
       </c>
       <c r="G874" s="13" t="inlineStr"/>
@@ -44889,22 +44889,22 @@
       </c>
       <c r="C875" s="15" t="inlineStr">
         <is>
-          <t>Paso 3 · quiénes van</t>
+          <t>Paso 3</t>
         </is>
       </c>
       <c r="D875" s="15" t="inlineStr">
         <is>
-          <t>Texto</t>
+          <t>Error</t>
         </is>
       </c>
       <c r="E875" s="15" t="inlineStr">
         <is>
-          <t>Grupo nuevo</t>
+          <t>Siguiente sin nadie</t>
         </is>
       </c>
       <c r="F875" s="15" t="inlineStr">
         <is>
-          <t>Se proponen las N personas que más esperan, primero las prioritarias y las de una misma institución de gobierno juntas. Quite o agregue a quien haga falta.</t>
+          <t>Elija a quién va · Marque la casilla junto al nombre de al menos una persona. El grupo se confirma con al menos 5.</t>
         </is>
       </c>
       <c r="G875" s="13" t="inlineStr"/>
@@ -44939,22 +44939,22 @@
       </c>
       <c r="C876" s="12" t="inlineStr">
         <is>
-          <t>Paso 3 · quiénes van</t>
+          <t>Paso 4 · confirmar</t>
         </is>
       </c>
       <c r="D876" s="12" t="inlineStr">
         <is>
-          <t>Texto</t>
+          <t>Estado</t>
         </is>
       </c>
       <c r="E876" s="12" t="inlineStr">
         <is>
-          <t>Siempre</t>
+          <t>Antes de crearlo</t>
         </is>
       </c>
       <c r="F876" s="12" t="inlineStr">
         <is>
-          <t>N de 25 lugares · se confirma con al menos 5 personas</t>
+          <t>Se crea confirmado · Cada persona verá en «Mis trámites» la fecha, la hora y el lugar. / Se crea por confirmar · Para confirmarlo le falta …</t>
         </is>
       </c>
       <c r="G876" s="13" t="inlineStr"/>
@@ -44989,22 +44989,22 @@
       </c>
       <c r="C877" s="15" t="inlineStr">
         <is>
-          <t>Paso 3 · quiénes van</t>
+          <t>Paso 4 · confirmar</t>
         </is>
       </c>
       <c r="D877" s="15" t="inlineStr">
         <is>
-          <t>Plegable</t>
+          <t>Botón</t>
         </is>
       </c>
       <c r="E877" s="15" t="inlineStr">
         <is>
-          <t>Con más en espera que las propuestas</t>
+          <t>Grupo nuevo</t>
         </is>
       </c>
       <c r="F877" s="15" t="inlineStr">
         <is>
-          <t>Cambiar a quiénes van (N más en espera)</t>
+          <t>Crear el grupo · Crear sin confirmar (sólo si podría confirmarse)</t>
         </is>
       </c>
       <c r="G877" s="13" t="inlineStr"/>
@@ -45039,22 +45039,22 @@
       </c>
       <c r="C878" s="12" t="inlineStr">
         <is>
-          <t>Paso 3</t>
+          <t>Paso 4 · confirmar</t>
         </is>
       </c>
       <c r="D878" s="12" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Botón</t>
         </is>
       </c>
       <c r="E878" s="12" t="inlineStr">
         <is>
-          <t>Siguiente sin nadie</t>
+          <t>Grupo que ya existe</t>
         </is>
       </c>
       <c r="F878" s="12" t="inlineStr">
         <is>
-          <t>Elija a quién va · Marque la casilla junto al nombre de al menos una persona. El grupo se confirma con al menos 5.</t>
+          <t>Confirmar el grupo / Guardar los cambios / Guardar sin confirmar / Agregar al grupo (confirmado)</t>
         </is>
       </c>
       <c r="G878" s="13" t="inlineStr"/>
@@ -45089,22 +45089,22 @@
       </c>
       <c r="C879" s="15" t="inlineStr">
         <is>
-          <t>Paso 4 · confirmar</t>
+          <t>Paso 4 · instructor</t>
         </is>
       </c>
       <c r="D879" s="15" t="inlineStr">
         <is>
-          <t>Estado</t>
+          <t>Ayuda (cambia)</t>
         </is>
       </c>
       <c r="E879" s="15" t="inlineStr">
         <is>
-          <t>Antes de crearlo</t>
+          <t>Instructor «Por asignar»</t>
         </is>
       </c>
       <c r="F879" s="15" t="inlineStr">
         <is>
-          <t>Se crea confirmado · Cada persona verá en «Mis trámites» la fecha, la hora y el lugar. / Se crea por confirmar · Para confirmarlo le falta …</t>
+          <t>Por asignar: el grupo se crea, pero no se confirma sin instructor. La asignación de instructores la hará el área de capacitación (pendiente P92).</t>
         </is>
       </c>
       <c r="G879" s="13" t="inlineStr"/>
@@ -45139,22 +45139,22 @@
       </c>
       <c r="C880" s="12" t="inlineStr">
         <is>
-          <t>Paso 4 · confirmar</t>
+          <t>Grupos programados</t>
         </is>
       </c>
       <c r="D880" s="12" t="inlineStr">
         <is>
-          <t>Botón</t>
+          <t>Aviso</t>
         </is>
       </c>
       <c r="E880" s="12" t="inlineStr">
         <is>
-          <t>Grupo nuevo</t>
+          <t>Al crear un grupo</t>
         </is>
       </c>
       <c r="F880" s="12" t="inlineStr">
         <is>
-          <t>Crear el grupo · Crear sin confirmar (sólo si podría confirmarse)</t>
+          <t>Grupo creado y confirmado: NOMBRE / Grupo creado, por confirmar: NOMBRE · FOLIO · N personas · entrada a las 09:00 · INSTRUCTOR. · Ver la ficha del grupo · Qué sigue</t>
         </is>
       </c>
       <c r="G880" s="13" t="inlineStr"/>
@@ -45189,22 +45189,22 @@
       </c>
       <c r="C881" s="15" t="inlineStr">
         <is>
-          <t>Paso 4 · confirmar</t>
+          <t>Grupos programados</t>
         </is>
       </c>
       <c r="D881" s="15" t="inlineStr">
         <is>
-          <t>Botón</t>
+          <t>Estado</t>
         </is>
       </c>
       <c r="E881" s="15" t="inlineStr">
         <is>
-          <t>Grupo que ya existe</t>
+          <t>Situación de cada grupo</t>
         </is>
       </c>
       <c r="F881" s="15" t="inlineStr">
         <is>
-          <t>Confirmar el grupo / Guardar los cambios / Guardar sin confirmar / Agregar al grupo (confirmado)</t>
+          <t>En curso · día N de 5 / Confirmado / Por confirmar / Sin semana / Propuesta vencida / Confirmado · no inició</t>
         </is>
       </c>
       <c r="G881" s="13" t="inlineStr"/>
@@ -45239,22 +45239,22 @@
       </c>
       <c r="C882" s="12" t="inlineStr">
         <is>
-          <t>Paso 4 · instructor</t>
+          <t>Grupos programados</t>
         </is>
       </c>
       <c r="D882" s="12" t="inlineStr">
         <is>
-          <t>Ayuda (cambia)</t>
+          <t>Botón o enlace</t>
         </is>
       </c>
       <c r="E882" s="12" t="inlineStr">
         <is>
-          <t>Instructor «Por asignar»</t>
+          <t>Acciones de cada grupo</t>
         </is>
       </c>
       <c r="F882" s="12" t="inlineStr">
         <is>
-          <t>Por asignar: el grupo se crea, pero no se confirma sin instructor. La asignación de instructores la hará el área de capacitación (pendiente P92).</t>
+          <t>Completar con las N que más esperan · Confirmar el grupo · Elegir semana / Cambiar la semana / Elegir otra semana · Agregar personas</t>
         </is>
       </c>
       <c r="G882" s="13" t="inlineStr"/>
@@ -45294,17 +45294,17 @@
       </c>
       <c r="D883" s="15" t="inlineStr">
         <is>
-          <t>Aviso</t>
+          <t>Texto</t>
         </is>
       </c>
       <c r="E883" s="15" t="inlineStr">
         <is>
-          <t>Al crear un grupo</t>
+          <t>Lo que falta</t>
         </is>
       </c>
       <c r="F883" s="15" t="inlineStr">
         <is>
-          <t>Grupo creado y confirmado: NOMBRE / Grupo creado, por confirmar: NOMBRE · FOLIO · N personas · entrada a las 09:00 · INSTRUCTOR. · Ver la ficha del grupo · Qué sigue</t>
+          <t>Semana, N personas, hora e instructor / Confirmarlo / —</t>
         </is>
       </c>
       <c r="G883" s="13" t="inlineStr"/>
@@ -45326,159 +45326,9 @@
         </is>
       </c>
     </row>
-    <row r="884">
-      <c r="A884" s="12" t="inlineStr">
-        <is>
-          <t>T883</t>
-        </is>
-      </c>
-      <c r="B884" s="12" t="inlineStr">
-        <is>
-          <t>Grupos (personal)</t>
-        </is>
-      </c>
-      <c r="C884" s="12" t="inlineStr">
-        <is>
-          <t>Grupos programados</t>
-        </is>
-      </c>
-      <c r="D884" s="12" t="inlineStr">
-        <is>
-          <t>Estado</t>
-        </is>
-      </c>
-      <c r="E884" s="12" t="inlineStr">
-        <is>
-          <t>Situación de cada grupo</t>
-        </is>
-      </c>
-      <c r="F884" s="12" t="inlineStr">
-        <is>
-          <t>En curso · día N de 5 / Confirmado / Por confirmar / Sin semana / Propuesta vencida / Confirmado · no inició</t>
-        </is>
-      </c>
-      <c r="G884" s="13" t="inlineStr"/>
-      <c r="H884" s="13" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="I884" s="13" t="inlineStr"/>
-      <c r="J884" s="12" t="inlineStr"/>
-      <c r="K884" s="14" t="inlineStr">
-        <is>
-          <t>Personal de la Secretaría</t>
-        </is>
-      </c>
-      <c r="L884" s="14" t="inlineStr">
-        <is>
-          <t>Código del sitio (sitio/app/grupos.js)</t>
-        </is>
-      </c>
-    </row>
-    <row r="885">
-      <c r="A885" s="15" t="inlineStr">
-        <is>
-          <t>T884</t>
-        </is>
-      </c>
-      <c r="B885" s="15" t="inlineStr">
-        <is>
-          <t>Grupos (personal)</t>
-        </is>
-      </c>
-      <c r="C885" s="15" t="inlineStr">
-        <is>
-          <t>Grupos programados</t>
-        </is>
-      </c>
-      <c r="D885" s="15" t="inlineStr">
-        <is>
-          <t>Botón o enlace</t>
-        </is>
-      </c>
-      <c r="E885" s="15" t="inlineStr">
-        <is>
-          <t>Acciones de cada grupo</t>
-        </is>
-      </c>
-      <c r="F885" s="15" t="inlineStr">
-        <is>
-          <t>Completar con las N que más esperan · Confirmar el grupo · Elegir semana / Cambiar la semana / Elegir otra semana · Agregar personas</t>
-        </is>
-      </c>
-      <c r="G885" s="13" t="inlineStr"/>
-      <c r="H885" s="13" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="I885" s="13" t="inlineStr"/>
-      <c r="J885" s="15" t="inlineStr"/>
-      <c r="K885" s="16" t="inlineStr">
-        <is>
-          <t>Personal de la Secretaría</t>
-        </is>
-      </c>
-      <c r="L885" s="16" t="inlineStr">
-        <is>
-          <t>Código del sitio (sitio/app/grupos.js)</t>
-        </is>
-      </c>
-    </row>
-    <row r="886">
-      <c r="A886" s="12" t="inlineStr">
-        <is>
-          <t>T885</t>
-        </is>
-      </c>
-      <c r="B886" s="12" t="inlineStr">
-        <is>
-          <t>Grupos (personal)</t>
-        </is>
-      </c>
-      <c r="C886" s="12" t="inlineStr">
-        <is>
-          <t>Grupos programados</t>
-        </is>
-      </c>
-      <c r="D886" s="12" t="inlineStr">
-        <is>
-          <t>Texto</t>
-        </is>
-      </c>
-      <c r="E886" s="12" t="inlineStr">
-        <is>
-          <t>Lo que falta</t>
-        </is>
-      </c>
-      <c r="F886" s="12" t="inlineStr">
-        <is>
-          <t>Semana, N personas, hora e instructor / Confirmarlo / —</t>
-        </is>
-      </c>
-      <c r="G886" s="13" t="inlineStr"/>
-      <c r="H886" s="13" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="I886" s="13" t="inlineStr"/>
-      <c r="J886" s="12" t="inlineStr"/>
-      <c r="K886" s="14" t="inlineStr">
-        <is>
-          <t>Personal de la Secretaría</t>
-        </is>
-      </c>
-      <c r="L886" s="14" t="inlineStr">
-        <is>
-          <t>Código del sitio (sitio/app/grupos.js)</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:L886"/>
-  <conditionalFormatting sqref="H2:H886">
+  <autoFilter ref="A1:L883"/>
+  <conditionalFormatting sqref="H2:H883">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"OK"</formula>
     </cfRule>
@@ -45492,13 +45342,13 @@
       <formula>"Duda"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G886">
+  <conditionalFormatting sqref="G2:G883">
     <cfRule type="expression" priority="5" dxfId="4">
       <formula>AND(LEN(G2)&gt;0,H2="Pendiente")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H886" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Estado" error="Elige: Pendiente, OK, Cambiar, Quitar o Duda." type="list">
+    <dataValidation sqref="H2:H883" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Estado" error="Elige: Pendiente, OK, Cambiar, Quitar o Duda." type="list">
       <formula1>"Pendiente,OK,Cambiar,Quitar,Duda"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Inventario de textos: ayuda de la carrera
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YEpbunHXM4tST7Mz5ceBJ7
</commit_message>
<xml_diff>
--- a/docs/textos/inventario-textos.xlsx
+++ b/docs/textos/inventario-textos.xlsx
@@ -600,7 +600,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Inventario generado de la versión de prueba 0.68 · 882 textos</t>
+          <t>Inventario generado de la versión de prueba 0.69 · 882 textos</t>
         </is>
       </c>
     </row>
@@ -15326,7 +15326,7 @@
       </c>
       <c r="F284" s="12" t="inlineStr">
         <is>
-          <t>Al escribir aparecen las ya registradas. Escribe la de tu posgrado (por ejemplo, Ciencias Forestales): cuenta aunque tu licenciatura sea de otra área.</t>
+          <t>Al escribir aparecen las ya registradas. Si la tuya no aparece, escríbela completa, como viene en tu título o cédula: la Secretaría la revisa. Escribe la de tu posgrado (por ejemplo, Ciencias Forestales): cuenta aunque tu licenciatura sea de otra área.</t>
         </is>
       </c>
       <c r="G284" s="13" t="inlineStr"/>

</xml_diff>

<commit_message>
Registro asistido y oportunidades para corregir: aviso por teléfono S7 y cuántas quedan
La solicitud de una persona del registro asistido que se cierra al agotar las
oportunidades de corrección deja su aviso por teléfono (S7, con el motivo); el
aviso S2 y la ventanilla dicen cuántas oportunidades le quedan o que es la
última, y la ventanilla dice qué pasó con la cerrada. Pruebas: probar-reglas
(S7 con el motivo, sin S4) y probar-sitio SOLO=asistido (avisos y ventanilla en
teléfono y computadora, con axe). REGLAS e inventario de textos al día.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YEpbunHXM4tST7Mz5ceBJ7
</commit_message>
<xml_diff>
--- a/docs/textos/inventario-textos.xlsx
+++ b/docs/textos/inventario-textos.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Textos" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Textos'!$A$1:$L$1003</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Textos'!$A$1:$L$1004</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -600,7 +600,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Inventario generado de la versión de prueba 0.69 · 1002 textos</t>
+          <t>Inventario generado de la versión de prueba 0.69 · 1003 textos</t>
         </is>
       </c>
     </row>
@@ -761,23 +761,23 @@
         </is>
       </c>
       <c r="B21" s="8">
-        <f>COUNTIF(Textos!$B$2:$B$1003,A21)</f>
+        <f>COUNTIF(Textos!$B$2:$B$1004,A21)</f>
         <v/>
       </c>
       <c r="C21" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$1003,A21,Textos!$H$2:$H$1003,"Pendiente")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$1004,A21,Textos!$H$2:$H$1004,"Pendiente")</f>
         <v/>
       </c>
       <c r="D21" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$1003,A21,Textos!$H$2:$H$1003,"OK")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$1004,A21,Textos!$H$2:$H$1004,"OK")</f>
         <v/>
       </c>
       <c r="E21" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$1003,A21,Textos!$H$2:$H$1003,"Cambiar")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$1004,A21,Textos!$H$2:$H$1004,"Cambiar")</f>
         <v/>
       </c>
       <c r="F21" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$1003,A21,Textos!$H$2:$H$1003,"Quitar")+COUNTIFS(Textos!$B$2:$B$1003,A21,Textos!$H$2:$H$1003,"Duda")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$1004,A21,Textos!$H$2:$H$1004,"Quitar")+COUNTIFS(Textos!$B$2:$B$1004,A21,Textos!$H$2:$H$1004,"Duda")</f>
         <v/>
       </c>
     </row>
@@ -788,23 +788,23 @@
         </is>
       </c>
       <c r="B22" s="8">
-        <f>COUNTIF(Textos!$B$2:$B$1003,A22)</f>
+        <f>COUNTIF(Textos!$B$2:$B$1004,A22)</f>
         <v/>
       </c>
       <c r="C22" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$1003,A22,Textos!$H$2:$H$1003,"Pendiente")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$1004,A22,Textos!$H$2:$H$1004,"Pendiente")</f>
         <v/>
       </c>
       <c r="D22" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$1003,A22,Textos!$H$2:$H$1003,"OK")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$1004,A22,Textos!$H$2:$H$1004,"OK")</f>
         <v/>
       </c>
       <c r="E22" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$1003,A22,Textos!$H$2:$H$1003,"Cambiar")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$1004,A22,Textos!$H$2:$H$1004,"Cambiar")</f>
         <v/>
       </c>
       <c r="F22" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$1003,A22,Textos!$H$2:$H$1003,"Quitar")+COUNTIFS(Textos!$B$2:$B$1003,A22,Textos!$H$2:$H$1003,"Duda")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$1004,A22,Textos!$H$2:$H$1004,"Quitar")+COUNTIFS(Textos!$B$2:$B$1004,A22,Textos!$H$2:$H$1004,"Duda")</f>
         <v/>
       </c>
     </row>
@@ -815,23 +815,23 @@
         </is>
       </c>
       <c r="B23" s="8">
-        <f>COUNTIF(Textos!$B$2:$B$1003,A23)</f>
+        <f>COUNTIF(Textos!$B$2:$B$1004,A23)</f>
         <v/>
       </c>
       <c r="C23" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$1003,A23,Textos!$H$2:$H$1003,"Pendiente")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$1004,A23,Textos!$H$2:$H$1004,"Pendiente")</f>
         <v/>
       </c>
       <c r="D23" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$1003,A23,Textos!$H$2:$H$1003,"OK")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$1004,A23,Textos!$H$2:$H$1004,"OK")</f>
         <v/>
       </c>
       <c r="E23" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$1003,A23,Textos!$H$2:$H$1003,"Cambiar")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$1004,A23,Textos!$H$2:$H$1004,"Cambiar")</f>
         <v/>
       </c>
       <c r="F23" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$1003,A23,Textos!$H$2:$H$1003,"Quitar")+COUNTIFS(Textos!$B$2:$B$1003,A23,Textos!$H$2:$H$1003,"Duda")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$1004,A23,Textos!$H$2:$H$1004,"Quitar")+COUNTIFS(Textos!$B$2:$B$1004,A23,Textos!$H$2:$H$1004,"Duda")</f>
         <v/>
       </c>
     </row>
@@ -842,23 +842,23 @@
         </is>
       </c>
       <c r="B24" s="8">
-        <f>COUNTIF(Textos!$B$2:$B$1003,A24)</f>
+        <f>COUNTIF(Textos!$B$2:$B$1004,A24)</f>
         <v/>
       </c>
       <c r="C24" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$1003,A24,Textos!$H$2:$H$1003,"Pendiente")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$1004,A24,Textos!$H$2:$H$1004,"Pendiente")</f>
         <v/>
       </c>
       <c r="D24" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$1003,A24,Textos!$H$2:$H$1003,"OK")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$1004,A24,Textos!$H$2:$H$1004,"OK")</f>
         <v/>
       </c>
       <c r="E24" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$1003,A24,Textos!$H$2:$H$1003,"Cambiar")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$1004,A24,Textos!$H$2:$H$1004,"Cambiar")</f>
         <v/>
       </c>
       <c r="F24" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$1003,A24,Textos!$H$2:$H$1003,"Quitar")+COUNTIFS(Textos!$B$2:$B$1003,A24,Textos!$H$2:$H$1003,"Duda")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$1004,A24,Textos!$H$2:$H$1004,"Quitar")+COUNTIFS(Textos!$B$2:$B$1004,A24,Textos!$H$2:$H$1004,"Duda")</f>
         <v/>
       </c>
     </row>
@@ -869,23 +869,23 @@
         </is>
       </c>
       <c r="B25" s="8">
-        <f>COUNTIF(Textos!$B$2:$B$1003,A25)</f>
+        <f>COUNTIF(Textos!$B$2:$B$1004,A25)</f>
         <v/>
       </c>
       <c r="C25" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$1003,A25,Textos!$H$2:$H$1003,"Pendiente")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$1004,A25,Textos!$H$2:$H$1004,"Pendiente")</f>
         <v/>
       </c>
       <c r="D25" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$1003,A25,Textos!$H$2:$H$1003,"OK")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$1004,A25,Textos!$H$2:$H$1004,"OK")</f>
         <v/>
       </c>
       <c r="E25" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$1003,A25,Textos!$H$2:$H$1003,"Cambiar")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$1004,A25,Textos!$H$2:$H$1004,"Cambiar")</f>
         <v/>
       </c>
       <c r="F25" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$1003,A25,Textos!$H$2:$H$1003,"Quitar")+COUNTIFS(Textos!$B$2:$B$1003,A25,Textos!$H$2:$H$1003,"Duda")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$1004,A25,Textos!$H$2:$H$1004,"Quitar")+COUNTIFS(Textos!$B$2:$B$1004,A25,Textos!$H$2:$H$1004,"Duda")</f>
         <v/>
       </c>
     </row>
@@ -896,23 +896,23 @@
         </is>
       </c>
       <c r="B26" s="8">
-        <f>COUNTIF(Textos!$B$2:$B$1003,A26)</f>
+        <f>COUNTIF(Textos!$B$2:$B$1004,A26)</f>
         <v/>
       </c>
       <c r="C26" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$1003,A26,Textos!$H$2:$H$1003,"Pendiente")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$1004,A26,Textos!$H$2:$H$1004,"Pendiente")</f>
         <v/>
       </c>
       <c r="D26" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$1003,A26,Textos!$H$2:$H$1003,"OK")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$1004,A26,Textos!$H$2:$H$1004,"OK")</f>
         <v/>
       </c>
       <c r="E26" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$1003,A26,Textos!$H$2:$H$1003,"Cambiar")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$1004,A26,Textos!$H$2:$H$1004,"Cambiar")</f>
         <v/>
       </c>
       <c r="F26" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$1003,A26,Textos!$H$2:$H$1003,"Quitar")+COUNTIFS(Textos!$B$2:$B$1003,A26,Textos!$H$2:$H$1003,"Duda")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$1004,A26,Textos!$H$2:$H$1004,"Quitar")+COUNTIFS(Textos!$B$2:$B$1004,A26,Textos!$H$2:$H$1004,"Duda")</f>
         <v/>
       </c>
     </row>
@@ -923,23 +923,23 @@
         </is>
       </c>
       <c r="B27" s="8">
-        <f>COUNTIF(Textos!$B$2:$B$1003,A27)</f>
+        <f>COUNTIF(Textos!$B$2:$B$1004,A27)</f>
         <v/>
       </c>
       <c r="C27" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$1003,A27,Textos!$H$2:$H$1003,"Pendiente")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$1004,A27,Textos!$H$2:$H$1004,"Pendiente")</f>
         <v/>
       </c>
       <c r="D27" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$1003,A27,Textos!$H$2:$H$1003,"OK")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$1004,A27,Textos!$H$2:$H$1004,"OK")</f>
         <v/>
       </c>
       <c r="E27" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$1003,A27,Textos!$H$2:$H$1003,"Cambiar")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$1004,A27,Textos!$H$2:$H$1004,"Cambiar")</f>
         <v/>
       </c>
       <c r="F27" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$1003,A27,Textos!$H$2:$H$1003,"Quitar")+COUNTIFS(Textos!$B$2:$B$1003,A27,Textos!$H$2:$H$1003,"Duda")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$1004,A27,Textos!$H$2:$H$1004,"Quitar")+COUNTIFS(Textos!$B$2:$B$1004,A27,Textos!$H$2:$H$1004,"Duda")</f>
         <v/>
       </c>
     </row>
@@ -950,23 +950,23 @@
         </is>
       </c>
       <c r="B28" s="8">
-        <f>COUNTIF(Textos!$B$2:$B$1003,A28)</f>
+        <f>COUNTIF(Textos!$B$2:$B$1004,A28)</f>
         <v/>
       </c>
       <c r="C28" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$1003,A28,Textos!$H$2:$H$1003,"Pendiente")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$1004,A28,Textos!$H$2:$H$1004,"Pendiente")</f>
         <v/>
       </c>
       <c r="D28" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$1003,A28,Textos!$H$2:$H$1003,"OK")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$1004,A28,Textos!$H$2:$H$1004,"OK")</f>
         <v/>
       </c>
       <c r="E28" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$1003,A28,Textos!$H$2:$H$1003,"Cambiar")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$1004,A28,Textos!$H$2:$H$1004,"Cambiar")</f>
         <v/>
       </c>
       <c r="F28" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$1003,A28,Textos!$H$2:$H$1003,"Quitar")+COUNTIFS(Textos!$B$2:$B$1003,A28,Textos!$H$2:$H$1003,"Duda")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$1004,A28,Textos!$H$2:$H$1004,"Quitar")+COUNTIFS(Textos!$B$2:$B$1004,A28,Textos!$H$2:$H$1004,"Duda")</f>
         <v/>
       </c>
     </row>
@@ -977,23 +977,23 @@
         </is>
       </c>
       <c r="B29" s="8">
-        <f>COUNTIF(Textos!$B$2:$B$1003,A29)</f>
+        <f>COUNTIF(Textos!$B$2:$B$1004,A29)</f>
         <v/>
       </c>
       <c r="C29" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$1003,A29,Textos!$H$2:$H$1003,"Pendiente")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$1004,A29,Textos!$H$2:$H$1004,"Pendiente")</f>
         <v/>
       </c>
       <c r="D29" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$1003,A29,Textos!$H$2:$H$1003,"OK")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$1004,A29,Textos!$H$2:$H$1004,"OK")</f>
         <v/>
       </c>
       <c r="E29" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$1003,A29,Textos!$H$2:$H$1003,"Cambiar")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$1004,A29,Textos!$H$2:$H$1004,"Cambiar")</f>
         <v/>
       </c>
       <c r="F29" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$1003,A29,Textos!$H$2:$H$1003,"Quitar")+COUNTIFS(Textos!$B$2:$B$1003,A29,Textos!$H$2:$H$1003,"Duda")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$1004,A29,Textos!$H$2:$H$1004,"Quitar")+COUNTIFS(Textos!$B$2:$B$1004,A29,Textos!$H$2:$H$1004,"Duda")</f>
         <v/>
       </c>
     </row>
@@ -1004,23 +1004,23 @@
         </is>
       </c>
       <c r="B30" s="8">
-        <f>COUNTIF(Textos!$B$2:$B$1003,A30)</f>
+        <f>COUNTIF(Textos!$B$2:$B$1004,A30)</f>
         <v/>
       </c>
       <c r="C30" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$1003,A30,Textos!$H$2:$H$1003,"Pendiente")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$1004,A30,Textos!$H$2:$H$1004,"Pendiente")</f>
         <v/>
       </c>
       <c r="D30" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$1003,A30,Textos!$H$2:$H$1003,"OK")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$1004,A30,Textos!$H$2:$H$1004,"OK")</f>
         <v/>
       </c>
       <c r="E30" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$1003,A30,Textos!$H$2:$H$1003,"Cambiar")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$1004,A30,Textos!$H$2:$H$1004,"Cambiar")</f>
         <v/>
       </c>
       <c r="F30" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$1003,A30,Textos!$H$2:$H$1003,"Quitar")+COUNTIFS(Textos!$B$2:$B$1003,A30,Textos!$H$2:$H$1003,"Duda")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$1004,A30,Textos!$H$2:$H$1004,"Quitar")+COUNTIFS(Textos!$B$2:$B$1004,A30,Textos!$H$2:$H$1004,"Duda")</f>
         <v/>
       </c>
     </row>
@@ -1031,23 +1031,23 @@
         </is>
       </c>
       <c r="B31" s="8">
-        <f>COUNTIF(Textos!$B$2:$B$1003,A31)</f>
+        <f>COUNTIF(Textos!$B$2:$B$1004,A31)</f>
         <v/>
       </c>
       <c r="C31" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$1003,A31,Textos!$H$2:$H$1003,"Pendiente")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$1004,A31,Textos!$H$2:$H$1004,"Pendiente")</f>
         <v/>
       </c>
       <c r="D31" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$1003,A31,Textos!$H$2:$H$1003,"OK")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$1004,A31,Textos!$H$2:$H$1004,"OK")</f>
         <v/>
       </c>
       <c r="E31" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$1003,A31,Textos!$H$2:$H$1003,"Cambiar")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$1004,A31,Textos!$H$2:$H$1004,"Cambiar")</f>
         <v/>
       </c>
       <c r="F31" s="8">
-        <f>COUNTIFS(Textos!$B$2:$B$1003,A31,Textos!$H$2:$H$1003,"Quitar")+COUNTIFS(Textos!$B$2:$B$1003,A31,Textos!$H$2:$H$1003,"Duda")</f>
+        <f>COUNTIFS(Textos!$B$2:$B$1004,A31,Textos!$H$2:$H$1004,"Quitar")+COUNTIFS(Textos!$B$2:$B$1004,A31,Textos!$H$2:$H$1004,"Duda")</f>
         <v/>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1003"/>
+  <dimension ref="A1:L1004"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -50762,7 +50762,7 @@
       </c>
       <c r="F992" s="12" t="inlineStr">
         <is>
-          <t>Solicitud con observaciones · Cerrada por no corregir a tiempo · Cita de cotejo · Solicitud rechazada · Resultado de la cita de cotejo · Cuenta bloqueada por identidad · Grupo asignado · Cambio en su grupo · Resultado del examen · Acreditación entregada · Acreditación cancelada · Reposición de la credencial</t>
+          <t>Solicitud con observaciones · Cerrada por no corregir a tiempo · Cita de cotejo · Solicitud rechazada · Cerrada: sin más oportunidades de corrección · Resultado de la cita de cotejo · Cuenta bloqueada por identidad · Grupo asignado · Cambio en su grupo · Resultado del examen · Acreditación entregada · Acreditación cancelada · Reposición de la credencial</t>
         </is>
       </c>
       <c r="G992" s="13" t="inlineStr"/>
@@ -50812,7 +50812,7 @@
       </c>
       <c r="F993" s="15" t="inlineStr">
         <is>
-          <t>A tu solicitud FOLIO le falta corregir algo: DOCUMENTOS. Ven a la ventanilla del SEDE, HORARIO, para que te digamos qué falta y lo corrijamos contigo. Hay un plazo para corregir.</t>
+          <t>A tu solicitud FOLIO le falta corregir algo: DOCUMENTOS. Ven a la ventanilla del SEDE, HORARIO, para que te digamos qué falta y lo corrijamos contigo. Hay un plazo para corregir. Te quedan N oportunidades para corregir. / Esta es tu última oportunidad para corregir. Si en la revisión siguen las observaciones, tu solicitud se cierra y tienes que iniciar una nueva.</t>
         </is>
       </c>
       <c r="G993" s="13" t="inlineStr"/>
@@ -50857,12 +50857,12 @@
       </c>
       <c r="E994" s="12" t="inlineStr">
         <is>
-          <t>Cita de cotejo</t>
+          <t>Cerrada al agotar las oportunidades de corrección</t>
         </is>
       </c>
       <c r="F994" s="12" t="inlineStr">
         <is>
-          <t>Tus documentos están completos. Tu cita de cotejo es el DÍA a las HH:MM, en el SEDE. Lleva los mismos documentos impresos, tu identificación oficial y el comprobante del pago de $MONTO con la referencia REFERENCIA.</t>
+          <t>Tu solicitud FOLIO se cerró porque, después de tu última oportunidad para corregir, tus documentos siguieron con observaciones. No pagaste nada y puedes iniciar una solicitud nueva en la ventanilla del SEDE, HORARIO.</t>
         </is>
       </c>
       <c r="G994" s="13" t="inlineStr"/>
@@ -50907,12 +50907,12 @@
       </c>
       <c r="E995" s="15" t="inlineStr">
         <is>
-          <t>Resultado de la cita</t>
+          <t>Cita de cotejo</t>
         </is>
       </c>
       <c r="F995" s="15" t="inlineStr">
         <is>
-          <t>Tu cotejo terminó; tu expediente es el EXP-… / En tu cita faltó un documento: …; tráelo hoy mismo … / En tu cita, un documento no coincidió … / Como no llegaste a tu cita (o no llevaste el comprobante de pago), te dimos una cita nueva: … / Tu solicitud FOLIO se cerró porque no llegaste dos veces a tu cita de cotejo.</t>
+          <t>Tus documentos están completos. Tu cita de cotejo es el DÍA a las HH:MM, en el SEDE. Lleva los mismos documentos impresos, tu identificación oficial y el comprobante del pago de $MONTO con la referencia REFERENCIA.</t>
         </is>
       </c>
       <c r="G995" s="13" t="inlineStr"/>
@@ -50957,12 +50957,12 @@
       </c>
       <c r="E996" s="12" t="inlineStr">
         <is>
-          <t>Otros avisos</t>
+          <t>Resultado de la cita</t>
         </is>
       </c>
       <c r="F996" s="12" t="inlineStr">
         <is>
-          <t>Cerrada sin corregir · Rechazada (con el motivo) · Cuenta bloqueada · Grupo asignado (día, hora y sede) · Baja, cambio o grupo por confirmar · Resultado del examen · Acreditación entregada o cancelada · Reposición de la credencial</t>
+          <t>Tu cotejo terminó; tu expediente es el EXP-… / En tu cita faltó un documento: …; tráelo hoy mismo … / En tu cita, un documento no coincidió … / Como no llegaste a tu cita (o no llevaste el comprobante de pago), te dimos una cita nueva: … / Tu solicitud FOLIO se cerró porque no llegaste dos veces a tu cita de cotejo.</t>
         </is>
       </c>
       <c r="G996" s="13" t="inlineStr"/>
@@ -50997,22 +50997,22 @@
       </c>
       <c r="C997" s="15" t="inlineStr">
         <is>
-          <t>Al registrar</t>
+          <t>Qué decirle (de tú)</t>
         </is>
       </c>
       <c r="D997" s="15" t="inlineStr">
         <is>
-          <t>Aviso</t>
+          <t>Texto</t>
         </is>
       </c>
       <c r="E997" s="15" t="inlineStr">
         <is>
-          <t>Resultado</t>
+          <t>Otros avisos</t>
         </is>
       </c>
       <c r="F997" s="15" t="inlineStr">
         <is>
-          <t>Se registró que se le avisó · NOMBRE: aviso hecho. / Se registró que no contestó · NOMBRE no contestó. Lo que se le iba a decir se le dice cuando vaya a la ventanilla. / Ya estaba registrado · Otra persona del personal ya registró el aviso de NOMBRE.</t>
+          <t>Cerrada sin corregir · Rechazada (con el motivo) · Cuenta bloqueada · Grupo asignado (día, hora y sede) · Baja, cambio o grupo por confirmar · Resultado del examen · Acreditación entregada o cancelada · Reposición de la credencial</t>
         </is>
       </c>
       <c r="G997" s="13" t="inlineStr"/>
@@ -51042,27 +51042,27 @@
       </c>
       <c r="B998" s="12" t="inlineStr">
         <is>
-          <t>Revisar una solicitud y Cita de cotejo (personal)</t>
+          <t>Inicio del personal · avisos por teléfono</t>
         </is>
       </c>
       <c r="C998" s="12" t="inlineStr">
         <is>
-          <t>Cabecera</t>
+          <t>Al registrar</t>
         </is>
       </c>
       <c r="D998" s="12" t="inlineStr">
         <is>
-          <t>Estado</t>
+          <t>Aviso</t>
         </is>
       </c>
       <c r="E998" s="12" t="inlineStr">
         <is>
-          <t>Persona del registro asistido sin activar</t>
+          <t>Resultado</t>
         </is>
       </c>
       <c r="F998" s="12" t="inlineStr">
         <is>
-          <t>Registro asistido: avisar por teléfono, 55 1234 5678</t>
+          <t>Se registró que se le avisó · NOMBRE: aviso hecho. / Se registró que no contestó · NOMBRE no contestó. Lo que se le iba a decir se le dice cuando vaya a la ventanilla. / Ya estaba registrado · Otra persona del personal ya registró el aviso de NOMBRE.</t>
         </is>
       </c>
       <c r="G998" s="13" t="inlineStr"/>
@@ -51092,27 +51092,27 @@
       </c>
       <c r="B999" s="15" t="inlineStr">
         <is>
-          <t>Ventanilla (personal)</t>
+          <t>Revisar una solicitud y Cita de cotejo (personal)</t>
         </is>
       </c>
       <c r="C999" s="15" t="inlineStr">
         <is>
-          <t>Búsqueda</t>
+          <t>Cabecera</t>
         </is>
       </c>
       <c r="D999" s="15" t="inlineStr">
         <is>
-          <t>Texto</t>
+          <t>Estado</t>
         </is>
       </c>
       <c r="E999" s="15" t="inlineStr">
         <is>
-          <t>Al buscar</t>
+          <t>Persona del registro asistido sin activar</t>
         </is>
       </c>
       <c r="F999" s="15" t="inlineStr">
         <is>
-          <t>Escriba al menos 3 caracteres para buscar. / N personas encontradas. / Nadie coincide con la búsqueda. Revise lo que escribió.</t>
+          <t>Registro asistido: avisar por teléfono, 55 1234 5678</t>
         </is>
       </c>
       <c r="G999" s="13" t="inlineStr"/>
@@ -51130,7 +51130,7 @@
       </c>
       <c r="L999" s="16" t="inlineStr">
         <is>
-          <t>Código del sitio (sitio/app/ventanilla.js)</t>
+          <t>Código del sitio (sitio/app/registro-asistido.js)</t>
         </is>
       </c>
     </row>
@@ -51147,22 +51147,22 @@
       </c>
       <c r="C1000" s="12" t="inlineStr">
         <is>
-          <t>Ficha</t>
+          <t>Búsqueda</t>
         </is>
       </c>
       <c r="D1000" s="12" t="inlineStr">
         <is>
-          <t>Estado</t>
+          <t>Texto</t>
         </is>
       </c>
       <c r="E1000" s="12" t="inlineStr">
         <is>
-          <t>Según la cuenta</t>
+          <t>Al buscar</t>
         </is>
       </c>
       <c r="F1000" s="12" t="inlineStr">
         <is>
-          <t>Registro asistido · avisos por teléfono / Registro asistido · ya activó su cuenta / Registro anterior · sin cuenta en línea / Cuenta bloqueada / Cuenta en línea</t>
+          <t>Escriba al menos 3 caracteres para buscar. / N personas encontradas. / Nadie coincide con la búsqueda. Revise lo que escribió.</t>
         </is>
       </c>
       <c r="G1000" s="13" t="inlineStr"/>
@@ -51202,17 +51202,17 @@
       </c>
       <c r="D1001" s="15" t="inlineStr">
         <is>
-          <t>Aviso</t>
+          <t>Estado</t>
         </is>
       </c>
       <c r="E1001" s="15" t="inlineStr">
         <is>
-          <t>Con avisos por teléfono pendientes</t>
+          <t>Según la cuenta</t>
         </is>
       </c>
       <c r="F1001" s="15" t="inlineStr">
         <is>
-          <t>Tiene un aviso por teléfono pendiente (Tiene N avisos…) · Si está aquí, dígaselo y regístrelo en la lista de avisos por teléfono pendientes.</t>
+          <t>Registro asistido · avisos por teléfono / Registro asistido · ya activó su cuenta / Registro anterior · sin cuenta en línea / Cuenta bloqueada / Cuenta en línea</t>
         </is>
       </c>
       <c r="G1001" s="13" t="inlineStr"/>
@@ -51247,22 +51247,22 @@
       </c>
       <c r="C1002" s="12" t="inlineStr">
         <is>
-          <t>Ficha · Qué decirle (de tú)</t>
+          <t>Ficha</t>
         </is>
       </c>
       <c r="D1002" s="12" t="inlineStr">
         <is>
-          <t>Texto</t>
+          <t>Aviso</t>
         </is>
       </c>
       <c r="E1002" s="12" t="inlineStr">
         <is>
-          <t>Según el estado</t>
+          <t>Con avisos por teléfono pendientes</t>
         </is>
       </c>
       <c r="F1002" s="12" t="inlineStr">
         <is>
-          <t>Tu solicitud todavía no se envía: falta terminar de capturarla contigo. / La Secretaría está revisando tus documentos. … / A tu solicitud le falta corregir un documento: … Lo corregimos aquí contigo. Hay un plazo para corregir. / Tu cita de cotejo es el … / Tu curso empieza el … / Tu cotejo terminó. Estás en espera de un grupo del curso … (y los «qué sigue» de «Mis trámites»)</t>
+          <t>Tiene un aviso por teléfono pendiente (Tiene N avisos…) · Si está aquí, dígaselo y regístrelo en la lista de avisos por teléfono pendientes.</t>
         </is>
       </c>
       <c r="G1002" s="13" t="inlineStr"/>
@@ -51280,7 +51280,7 @@
       </c>
       <c r="L1002" s="14" t="inlineStr">
         <is>
-          <t>Código del sitio (sitio/app/registro-asistido.js)</t>
+          <t>Código del sitio (sitio/app/ventanilla.js)</t>
         </is>
       </c>
     </row>
@@ -51297,22 +51297,22 @@
       </c>
       <c r="C1003" s="15" t="inlineStr">
         <is>
-          <t>Ficha</t>
+          <t>Ficha · Qué decirle (de tú)</t>
         </is>
       </c>
       <c r="D1003" s="15" t="inlineStr">
         <is>
-          <t>Botón o enlace</t>
+          <t>Texto</t>
         </is>
       </c>
       <c r="E1003" s="15" t="inlineStr">
         <is>
-          <t>Persona del registro asistido</t>
+          <t>Según el estado</t>
         </is>
       </c>
       <c r="F1003" s="15" t="inlineStr">
         <is>
-          <t>Leerle lo que falta y cargar lo corregido · Seguir capturando su solicitud · Capturar una solicitud nueva</t>
+          <t>Tu solicitud todavía no se envía: falta terminar de capturarla contigo. / La Secretaría está revisando tus documentos. … / A tu solicitud le falta corregir un documento: … Lo corregimos aquí contigo. Hay un plazo para corregir. Te quedan N oportunidades para corregir. (o: Esta es tu última oportunidad para corregir. …) / Tu solicitud se cerró porque, después de tu última oportunidad para corregir, tus documentos siguieron con observaciones. No pagaste nada y puedes iniciar una solicitud nueva aquí mismo. / Tu cita de cotejo es el … / Tu curso empieza el … / Tu cotejo terminó. Estás en espera de un grupo del curso … (y los «qué sigue» de «Mis trámites»)</t>
         </is>
       </c>
       <c r="G1003" s="13" t="inlineStr"/>
@@ -51330,13 +51330,63 @@
       </c>
       <c r="L1003" s="16" t="inlineStr">
         <is>
+          <t>Código del sitio (sitio/app/registro-asistido.js)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1004">
+      <c r="A1004" s="12" t="inlineStr">
+        <is>
+          <t>T1003</t>
+        </is>
+      </c>
+      <c r="B1004" s="12" t="inlineStr">
+        <is>
+          <t>Ventanilla (personal)</t>
+        </is>
+      </c>
+      <c r="C1004" s="12" t="inlineStr">
+        <is>
+          <t>Ficha</t>
+        </is>
+      </c>
+      <c r="D1004" s="12" t="inlineStr">
+        <is>
+          <t>Botón o enlace</t>
+        </is>
+      </c>
+      <c r="E1004" s="12" t="inlineStr">
+        <is>
+          <t>Persona del registro asistido</t>
+        </is>
+      </c>
+      <c r="F1004" s="12" t="inlineStr">
+        <is>
+          <t>Leerle lo que falta y cargar lo corregido · Seguir capturando su solicitud · Capturar una solicitud nueva</t>
+        </is>
+      </c>
+      <c r="G1004" s="13" t="inlineStr"/>
+      <c r="H1004" s="13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I1004" s="13" t="inlineStr"/>
+      <c r="J1004" s="12" t="inlineStr"/>
+      <c r="K1004" s="14" t="inlineStr">
+        <is>
+          <t>Personal de la Secretaría</t>
+        </is>
+      </c>
+      <c r="L1004" s="14" t="inlineStr">
+        <is>
           <t>Código del sitio (sitio/app/ventanilla.js)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L1003"/>
-  <conditionalFormatting sqref="H2:H1003">
+  <autoFilter ref="A1:L1004"/>
+  <conditionalFormatting sqref="H2:H1004">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"OK"</formula>
     </cfRule>
@@ -51350,13 +51400,13 @@
       <formula>"Duda"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G1003">
+  <conditionalFormatting sqref="G2:G1004">
     <cfRule type="expression" priority="5" dxfId="4">
       <formula>AND(LEN(G2)&gt;0,H2="Pendiente")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H1003" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Estado" error="Elige: Pendiente, OK, Cambiar, Quitar o Duda." type="list">
+    <dataValidation sqref="H2:H1004" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Estado" error="Elige: Pendiente, OK, Cambiar, Quitar o Duda." type="list">
       <formula1>"Pendiente,OK,Cambiar,Quitar,Duda"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Constancia de situación fiscal: enlace del SAT para generarla
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YEpbunHXM4tST7Mz5ceBJ7
</commit_message>
<xml_diff>
--- a/docs/textos/inventario-textos.xlsx
+++ b/docs/textos/inventario-textos.xlsx
@@ -600,7 +600,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Inventario generado de la versión de prueba 0.69 · 1003 textos</t>
+          <t>Inventario generado de la versión de prueba 0.70 · 1003 textos</t>
         </is>
       </c>
     </row>
@@ -14476,7 +14476,7 @@
       </c>
       <c r="F267" s="15" t="inlineStr">
         <is>
-          <t>Tuya, como persona solicitante, emitida en el mes en curso. De ella se toman tu nombre, tu régimen y tu domicilio fiscal para la factura del pago.</t>
+          <t>Tuya, como persona solicitante, emitida en el mes en curso. De ella se toman tu nombre, tu régimen y tu domicilio fiscal para la factura del pago. Cómo generar tu constancia de situación fiscal en el SAT.</t>
         </is>
       </c>
       <c r="G267" s="13" t="inlineStr"/>

</xml_diff>